<commit_message>
fix: update verificacion excel template
</commit_message>
<xml_diff>
--- a/app/templates/Template_Verificacion.xlsx
+++ b/app/templates/Template_Verificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526FCD07-07EB-458E-8C75-C5C3ABD33F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86957E45-3F63-46FA-A096-056A1C27578F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A76715E4-29FC-4532-A462-AEFC175FF6CC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="99">
   <si>
     <t>CÓDIGO:</t>
   </si>
@@ -391,9 +391,6 @@
     <t>VERIFICADO POR:</t>
   </si>
   <si>
-    <t>FECHA VERIFIC.:</t>
-  </si>
-  <si>
     <t>BUENA (capeo)</t>
   </si>
   <si>
@@ -429,12 +426,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">DIAMETRO </t>
-  </si>
-  <si>
-    <t>Aceptaciòn</t>
-  </si>
-  <si>
     <t>ACEPTACION</t>
   </si>
   <si>
@@ -442,22 +433,6 @@
   </si>
   <si>
     <t>Uso de escudra metálica de 90, con refuerzo y calibre de laina y/o Calibre de cuña Desviación de 3mm(30x15cm); 2mm (20x10cm)</t>
-  </si>
-  <si>
-    <t>SUP 1
-Aceptacion</t>
-  </si>
-  <si>
-    <t>SUP 2
-Aceptacion</t>
-  </si>
-  <si>
-    <t>INF 1
-Aceptacion</t>
-  </si>
-  <si>
-    <t>INF 2
-Aceptacion</t>
   </si>
   <si>
     <t>PERPENDICULARIDAD                                                                                    (4inx8in &lt; 2mm) o (6inx12in &lt; 3mm)</t>
@@ -472,30 +447,6 @@
   <si>
     <t>C. INFERIOR 
 &lt; 0.05 mm Aceptacion</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Depresiones
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>≤</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 5 mm Aceptacion</t>
-    </r>
   </si>
   <si>
     <t>(4inx8in &lt; 2mm) o (6inx12in &lt; 3mm) y Medida &lt; 0,5º</t>
@@ -577,9 +528,6 @@
     <t>Còdigo equipo</t>
   </si>
   <si>
-    <t>Bernier</t>
-  </si>
-  <si>
     <t>Lainas 1</t>
   </si>
   <si>
@@ -590,16 +538,77 @@
   </si>
   <si>
     <t>Balanza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÍAMETRO </t>
+  </si>
+  <si>
+    <t>Aceptación</t>
+  </si>
+  <si>
+    <t>SUP 1
+Aceptación</t>
+  </si>
+  <si>
+    <t>SUP 2
+Aceptación</t>
+  </si>
+  <si>
+    <t>INF 1
+Aceptación</t>
+  </si>
+  <si>
+    <t>INF 2
+Aceptación</t>
+  </si>
+  <si>
+    <t>C. SUPERIOR 
+&lt; 0.05 mm Aceptación</t>
+  </si>
+  <si>
+    <t>C. INFERIOR 
+&lt; 0.05 mm Aceptación</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Depresiones
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>≤</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 5 mm Aceptación</t>
+    </r>
+  </si>
+  <si>
+    <t>Vernier</t>
+  </si>
+  <si>
+    <t>FECHA DE VERIFICACIÓN.:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="&quot;0&quot;0"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="29" x14ac:knownFonts="1">
     <font>
@@ -1152,7 +1161,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="204">
+  <cellXfs count="205">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
@@ -1581,15 +1590,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1787,6 +1787,18 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1931,27 +1943,27 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>167640</xdr:colOff>
+      <xdr:colOff>80962</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>23812</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
+      <xdr:colOff>291912</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>137160</xdr:rowOff>
+      <xdr:rowOff>148494</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="153821" name="Imagen 3">
+        <xdr:cNvPr id="6" name="Imagen 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2785D793-2F89-1FF4-4835-26AE8D04290D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26436073-326F-4E5C-B848-D781FADBE968}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1962,42 +1974,18 @@
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="510540" y="38100"/>
-          <a:ext cx="990600" cy="579120"/>
+          <a:off x="423862" y="23812"/>
+          <a:ext cx="1025338" cy="610457"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -2568,111 +2556,107 @@
       <c r="A1" s="65"/>
       <c r="B1" s="66"/>
       <c r="C1" s="67"/>
-      <c r="D1" s="140" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="140"/>
-      <c r="F1" s="140"/>
-      <c r="G1" s="140"/>
-      <c r="H1" s="140"/>
-      <c r="I1" s="140"/>
-      <c r="J1" s="140"/>
-      <c r="K1" s="140"/>
-      <c r="L1" s="140"/>
-      <c r="M1" s="140"/>
-      <c r="N1" s="140"/>
-      <c r="O1" s="140"/>
-      <c r="P1" s="140"/>
-      <c r="Q1" s="140"/>
-      <c r="R1" s="30" t="s">
+      <c r="D1" s="137" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="137"/>
+      <c r="F1" s="137"/>
+      <c r="G1" s="137"/>
+      <c r="H1" s="137"/>
+      <c r="I1" s="137"/>
+      <c r="J1" s="137"/>
+      <c r="K1" s="137"/>
+      <c r="L1" s="137"/>
+      <c r="M1" s="137"/>
+      <c r="N1" s="137"/>
+      <c r="O1" s="137"/>
+      <c r="P1" s="137"/>
+      <c r="Q1" s="137"/>
+      <c r="T1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="S1" s="137" t="s">
+      <c r="U1" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="137"/>
-      <c r="U1" s="137"/>
+      <c r="V1" s="150"/>
     </row>
     <row r="2" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="68"/>
       <c r="B2" s="4"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="140"/>
-      <c r="E2" s="140"/>
-      <c r="F2" s="140"/>
-      <c r="G2" s="140"/>
-      <c r="H2" s="140"/>
-      <c r="I2" s="140"/>
-      <c r="J2" s="140"/>
-      <c r="K2" s="140"/>
-      <c r="L2" s="140"/>
-      <c r="M2" s="140"/>
-      <c r="N2" s="140"/>
-      <c r="O2" s="140"/>
-      <c r="P2" s="140"/>
-      <c r="Q2" s="140"/>
-      <c r="R2" s="19" t="s">
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="137"/>
+      <c r="H2" s="137"/>
+      <c r="I2" s="137"/>
+      <c r="J2" s="137"/>
+      <c r="K2" s="137"/>
+      <c r="L2" s="137"/>
+      <c r="M2" s="137"/>
+      <c r="N2" s="137"/>
+      <c r="O2" s="137"/>
+      <c r="P2" s="137"/>
+      <c r="Q2" s="137"/>
+      <c r="T2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="S2" s="138">
+      <c r="U2" s="201">
         <v>3</v>
       </c>
-      <c r="T2" s="138"/>
-      <c r="U2" s="138"/>
+      <c r="V2" s="202"/>
     </row>
     <row r="3" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="68"/>
       <c r="B3" s="4"/>
       <c r="C3" s="69"/>
-      <c r="D3" s="140"/>
-      <c r="E3" s="140"/>
-      <c r="F3" s="140"/>
-      <c r="G3" s="140"/>
-      <c r="H3" s="140"/>
-      <c r="I3" s="140"/>
-      <c r="J3" s="140"/>
-      <c r="K3" s="140"/>
-      <c r="L3" s="140"/>
-      <c r="M3" s="140"/>
-      <c r="N3" s="140"/>
-      <c r="O3" s="140"/>
-      <c r="P3" s="140"/>
-      <c r="Q3" s="140"/>
-      <c r="R3" s="19" t="s">
+      <c r="D3" s="137"/>
+      <c r="E3" s="137"/>
+      <c r="F3" s="137"/>
+      <c r="G3" s="137"/>
+      <c r="H3" s="137"/>
+      <c r="I3" s="137"/>
+      <c r="J3" s="137"/>
+      <c r="K3" s="137"/>
+      <c r="L3" s="137"/>
+      <c r="M3" s="137"/>
+      <c r="N3" s="137"/>
+      <c r="O3" s="137"/>
+      <c r="P3" s="137"/>
+      <c r="Q3" s="137"/>
+      <c r="T3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="S3" s="139">
+      <c r="U3" s="203">
         <v>46104</v>
       </c>
-      <c r="T3" s="139"/>
-      <c r="U3" s="139"/>
+      <c r="V3" s="204"/>
     </row>
     <row r="4" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="70"/>
       <c r="B4" s="71"/>
       <c r="C4" s="72"/>
-      <c r="D4" s="140"/>
-      <c r="E4" s="140"/>
-      <c r="F4" s="140"/>
-      <c r="G4" s="140"/>
-      <c r="H4" s="140"/>
-      <c r="I4" s="140"/>
-      <c r="J4" s="140"/>
-      <c r="K4" s="140"/>
-      <c r="L4" s="140"/>
-      <c r="M4" s="140"/>
-      <c r="N4" s="140"/>
-      <c r="O4" s="140"/>
-      <c r="P4" s="140"/>
-      <c r="Q4" s="140"/>
-      <c r="R4" s="30" t="s">
+      <c r="D4" s="137"/>
+      <c r="E4" s="137"/>
+      <c r="F4" s="137"/>
+      <c r="G4" s="137"/>
+      <c r="H4" s="137"/>
+      <c r="I4" s="137"/>
+      <c r="J4" s="137"/>
+      <c r="K4" s="137"/>
+      <c r="L4" s="137"/>
+      <c r="M4" s="137"/>
+      <c r="N4" s="137"/>
+      <c r="O4" s="137"/>
+      <c r="P4" s="137"/>
+      <c r="Q4" s="137"/>
+      <c r="T4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="S4" s="137" t="s">
+      <c r="U4" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="T4" s="137"/>
-      <c r="U4" s="137"/>
+      <c r="V4" s="150"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
@@ -2713,10 +2697,10 @@
       <c r="M6" s="134"/>
       <c r="N6" s="134"/>
       <c r="P6" s="76" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="Q6" s="88"/>
-      <c r="R6" s="1"/>
+      <c r="R6" s="88"/>
     </row>
     <row r="7" spans="1:22" ht="15.6" x14ac:dyDescent="0.25">
       <c r="A7" s="23"/>
@@ -2741,19 +2725,19 @@
         <v>5</v>
       </c>
       <c r="B8" s="128" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C8" s="130" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D8" s="118" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="E8" s="118"/>
       <c r="F8" s="118"/>
       <c r="G8" s="118"/>
       <c r="H8" s="119" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="I8" s="120"/>
       <c r="J8" s="120"/>
@@ -2765,18 +2749,18 @@
       <c r="N8" s="118"/>
       <c r="O8" s="118"/>
       <c r="P8" s="132" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="Q8" s="132" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="R8" s="122" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="S8" s="123"/>
       <c r="T8" s="124"/>
       <c r="U8" s="117" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="V8" s="117"/>
     </row>
@@ -2791,45 +2775,45 @@
         <v>37</v>
       </c>
       <c r="F9" s="77" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G9" s="63" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="H9" s="85" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="I9" s="85" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="J9" s="85" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="K9" s="85" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="L9" s="87" t="s">
         <v>41</v>
       </c>
       <c r="M9" s="86" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="N9" s="86" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="O9" s="86" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="P9" s="133"/>
       <c r="Q9" s="133"/>
       <c r="R9" s="87" t="s">
+        <v>55</v>
+      </c>
+      <c r="S9" s="87" t="s">
         <v>56</v>
       </c>
-      <c r="S9" s="87" t="s">
+      <c r="T9" s="87" t="s">
         <v>57</v>
-      </c>
-      <c r="T9" s="87" t="s">
-        <v>58</v>
       </c>
       <c r="U9" s="117"/>
       <c r="V9" s="117"/>
@@ -3029,26 +3013,26 @@
     <row r="18" spans="1:22" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="55"/>
       <c r="B18" s="113" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C18" s="113" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D18" s="21"/>
       <c r="E18" s="113" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="F18" s="21"/>
       <c r="G18" s="113" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="H18" s="21"/>
       <c r="I18" s="113" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="J18" s="21"/>
       <c r="K18" s="113" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="L18" s="21"/>
       <c r="M18" s="55"/>
@@ -3491,13 +3475,13 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="U2:V2"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="U4:V4"/>
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="C6:I6"/>
-    <mergeCell ref="S1:U1"/>
-    <mergeCell ref="S2:U2"/>
-    <mergeCell ref="S3:U3"/>
-    <mergeCell ref="S4:U4"/>
     <mergeCell ref="D1:Q4"/>
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="H7:L7"/>
@@ -3535,30 +3519,30 @@
   <sheetData>
     <row r="4" spans="2:5" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="92" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="93" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="93" t="s">
-        <v>63</v>
-      </c>
       <c r="D4" s="92" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E4" s="92" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="53.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="89" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="94" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="95" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" s="101" t="s">
         <v>80</v>
-      </c>
-      <c r="C5" s="94" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="95" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="101" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="73.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -3566,62 +3550,62 @@
         <v>19</v>
       </c>
       <c r="C6" s="97" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D6" s="89" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E6" s="96" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="141" t="s">
+      <c r="B7" s="138" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="142" t="s">
-        <v>75</v>
+      <c r="C7" s="139" t="s">
+        <v>68</v>
       </c>
       <c r="D7" s="98" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="141" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="138" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="141"/>
-      <c r="C8" s="142"/>
+      <c r="B8" s="138"/>
+      <c r="C8" s="139"/>
       <c r="D8" s="98" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="141"/>
+        <v>70</v>
+      </c>
+      <c r="E8" s="138"/>
     </row>
     <row r="9" spans="2:5" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="141"/>
-      <c r="C9" s="142"/>
+      <c r="B9" s="138"/>
+      <c r="C9" s="139"/>
       <c r="D9" s="98" t="s">
-        <v>82</v>
-      </c>
-      <c r="E9" s="141"/>
+        <v>74</v>
+      </c>
+      <c r="E9" s="138"/>
     </row>
     <row r="11" spans="2:5" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="99" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="99" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>27</v>
@@ -3665,110 +3649,110 @@
       <c r="A1" s="65"/>
       <c r="B1" s="66"/>
       <c r="C1" s="67"/>
-      <c r="D1" s="143" t="s">
+      <c r="D1" s="140" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="144"/>
-      <c r="F1" s="144"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="144"/>
-      <c r="I1" s="144"/>
-      <c r="J1" s="144"/>
-      <c r="K1" s="144"/>
-      <c r="L1" s="144"/>
-      <c r="M1" s="144"/>
-      <c r="N1" s="144"/>
-      <c r="O1" s="144"/>
-      <c r="P1" s="144"/>
-      <c r="Q1" s="145"/>
+      <c r="E1" s="141"/>
+      <c r="F1" s="141"/>
+      <c r="G1" s="141"/>
+      <c r="H1" s="141"/>
+      <c r="I1" s="141"/>
+      <c r="J1" s="141"/>
+      <c r="K1" s="141"/>
+      <c r="L1" s="141"/>
+      <c r="M1" s="141"/>
+      <c r="N1" s="141"/>
+      <c r="O1" s="141"/>
+      <c r="P1" s="141"/>
+      <c r="Q1" s="142"/>
       <c r="R1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="S1" s="152" t="s">
+      <c r="S1" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="153"/>
+      <c r="T1" s="150"/>
       <c r="U1" s="1"/>
     </row>
     <row r="2" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="68"/>
       <c r="B2" s="4"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="146"/>
-      <c r="E2" s="147"/>
-      <c r="F2" s="147"/>
-      <c r="G2" s="147"/>
-      <c r="H2" s="147"/>
-      <c r="I2" s="147"/>
-      <c r="J2" s="147"/>
-      <c r="K2" s="147"/>
-      <c r="L2" s="147"/>
-      <c r="M2" s="147"/>
-      <c r="N2" s="147"/>
-      <c r="O2" s="147"/>
-      <c r="P2" s="147"/>
-      <c r="Q2" s="148"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
+      <c r="K2" s="144"/>
+      <c r="L2" s="144"/>
+      <c r="M2" s="144"/>
+      <c r="N2" s="144"/>
+      <c r="O2" s="144"/>
+      <c r="P2" s="144"/>
+      <c r="Q2" s="145"/>
       <c r="R2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="S2" s="152">
+      <c r="S2" s="149">
         <v>1</v>
       </c>
-      <c r="T2" s="153"/>
+      <c r="T2" s="150"/>
       <c r="U2" s="1"/>
     </row>
     <row r="3" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="68"/>
       <c r="B3" s="4"/>
       <c r="C3" s="69"/>
-      <c r="D3" s="146"/>
-      <c r="E3" s="147"/>
-      <c r="F3" s="147"/>
-      <c r="G3" s="147"/>
-      <c r="H3" s="147"/>
-      <c r="I3" s="147"/>
-      <c r="J3" s="147"/>
-      <c r="K3" s="147"/>
-      <c r="L3" s="147"/>
-      <c r="M3" s="147"/>
-      <c r="N3" s="147"/>
-      <c r="O3" s="147"/>
-      <c r="P3" s="147"/>
-      <c r="Q3" s="148"/>
+      <c r="D3" s="143"/>
+      <c r="E3" s="144"/>
+      <c r="F3" s="144"/>
+      <c r="G3" s="144"/>
+      <c r="H3" s="144"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
+      <c r="M3" s="144"/>
+      <c r="N3" s="144"/>
+      <c r="O3" s="144"/>
+      <c r="P3" s="144"/>
+      <c r="Q3" s="145"/>
       <c r="R3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="S3" s="152">
+      <c r="S3" s="149">
         <v>45232</v>
       </c>
-      <c r="T3" s="153"/>
+      <c r="T3" s="150"/>
       <c r="U3" s="1"/>
     </row>
     <row r="4" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="70"/>
       <c r="B4" s="71"/>
       <c r="C4" s="72"/>
-      <c r="D4" s="149"/>
-      <c r="E4" s="150"/>
-      <c r="F4" s="150"/>
-      <c r="G4" s="150"/>
-      <c r="H4" s="150"/>
-      <c r="I4" s="150"/>
-      <c r="J4" s="150"/>
-      <c r="K4" s="150"/>
-      <c r="L4" s="150"/>
-      <c r="M4" s="150"/>
-      <c r="N4" s="150"/>
-      <c r="O4" s="150"/>
-      <c r="P4" s="150"/>
-      <c r="Q4" s="151"/>
+      <c r="D4" s="146"/>
+      <c r="E4" s="147"/>
+      <c r="F4" s="147"/>
+      <c r="G4" s="147"/>
+      <c r="H4" s="147"/>
+      <c r="I4" s="147"/>
+      <c r="J4" s="147"/>
+      <c r="K4" s="147"/>
+      <c r="L4" s="147"/>
+      <c r="M4" s="147"/>
+      <c r="N4" s="147"/>
+      <c r="O4" s="147"/>
+      <c r="P4" s="147"/>
+      <c r="Q4" s="148"/>
       <c r="R4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="S4" s="152" t="s">
+      <c r="S4" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="T4" s="153"/>
+      <c r="T4" s="150"/>
       <c r="U4" s="1"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -3801,16 +3785,16 @@
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
       <c r="D6" s="27"/>
-      <c r="E6" s="154"/>
-      <c r="F6" s="154"/>
+      <c r="E6" s="151"/>
+      <c r="F6" s="151"/>
       <c r="G6" s="28"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="155" t="s">
+      <c r="J6" s="152" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="155"/>
-      <c r="L6" s="155"/>
+      <c r="K6" s="152"/>
+      <c r="L6" s="152"/>
       <c r="M6" s="33"/>
       <c r="N6" s="52"/>
       <c r="O6" s="33"/>
@@ -3828,11 +3812,11 @@
       <c r="D7" s="18"/>
       <c r="E7" s="9"/>
       <c r="F7" s="10"/>
-      <c r="G7" s="156"/>
-      <c r="H7" s="156"/>
-      <c r="I7" s="156"/>
-      <c r="J7" s="156"/>
-      <c r="K7" s="156"/>
+      <c r="G7" s="153"/>
+      <c r="H7" s="153"/>
+      <c r="I7" s="153"/>
+      <c r="J7" s="153"/>
+      <c r="K7" s="153"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -3846,10 +3830,10 @@
       <c r="B8" s="23"/>
       <c r="C8" s="23"/>
       <c r="D8" s="29"/>
-      <c r="E8" s="157"/>
-      <c r="F8" s="157"/>
-      <c r="G8" s="157"/>
-      <c r="H8" s="157"/>
+      <c r="E8" s="154"/>
+      <c r="F8" s="154"/>
+      <c r="G8" s="154"/>
+      <c r="H8" s="154"/>
       <c r="I8" s="34"/>
       <c r="J8" s="34"/>
       <c r="K8" s="34"/>
@@ -3869,10 +3853,10 @@
       <c r="B9" s="23"/>
       <c r="C9" s="23"/>
       <c r="D9" s="29"/>
-      <c r="E9" s="157"/>
-      <c r="F9" s="157"/>
-      <c r="G9" s="157"/>
-      <c r="H9" s="157"/>
+      <c r="E9" s="154"/>
+      <c r="F9" s="154"/>
+      <c r="G9" s="154"/>
+      <c r="H9" s="154"/>
       <c r="I9" s="34"/>
       <c r="J9" s="34"/>
       <c r="K9" s="34"/>
@@ -3908,115 +3892,115 @@
       <c r="U10" s="1"/>
     </row>
     <row r="11" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="158" t="s">
+      <c r="A11" s="155" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="159" t="s">
+      <c r="B11" s="156" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="160" t="s">
+      <c r="C11" s="157" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="163" t="s">
+      <c r="D11" s="160" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="164"/>
-      <c r="F11" s="164"/>
-      <c r="G11" s="165"/>
-      <c r="H11" s="166" t="s">
+      <c r="E11" s="161"/>
+      <c r="F11" s="161"/>
+      <c r="G11" s="162"/>
+      <c r="H11" s="163" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="167"/>
-      <c r="J11" s="167"/>
-      <c r="K11" s="167"/>
-      <c r="L11" s="167"/>
-      <c r="M11" s="168" t="s">
+      <c r="I11" s="164"/>
+      <c r="J11" s="164"/>
+      <c r="K11" s="164"/>
+      <c r="L11" s="164"/>
+      <c r="M11" s="165" t="s">
         <v>18</v>
       </c>
-      <c r="N11" s="169"/>
-      <c r="O11" s="169"/>
-      <c r="P11" s="169"/>
-      <c r="Q11" s="169"/>
-      <c r="R11" s="170" t="s">
+      <c r="N11" s="166"/>
+      <c r="O11" s="166"/>
+      <c r="P11" s="166"/>
+      <c r="Q11" s="166"/>
+      <c r="R11" s="167" t="s">
         <v>34</v>
       </c>
-      <c r="S11" s="171"/>
-      <c r="T11" s="176" t="s">
+      <c r="S11" s="168"/>
+      <c r="T11" s="173" t="s">
         <v>33</v>
       </c>
       <c r="U11" s="1"/>
     </row>
     <row r="12" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="158"/>
-      <c r="B12" s="159"/>
-      <c r="C12" s="161"/>
-      <c r="D12" s="178" t="s">
+      <c r="A12" s="155"/>
+      <c r="B12" s="156"/>
+      <c r="C12" s="158"/>
+      <c r="D12" s="175" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="179"/>
-      <c r="F12" s="179"/>
-      <c r="G12" s="180"/>
-      <c r="H12" s="178" t="s">
+      <c r="E12" s="176"/>
+      <c r="F12" s="176"/>
+      <c r="G12" s="177"/>
+      <c r="H12" s="175" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="179"/>
-      <c r="J12" s="179"/>
-      <c r="K12" s="179"/>
-      <c r="L12" s="180"/>
-      <c r="M12" s="178" t="s">
+      <c r="I12" s="176"/>
+      <c r="J12" s="176"/>
+      <c r="K12" s="176"/>
+      <c r="L12" s="177"/>
+      <c r="M12" s="175" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="179"/>
-      <c r="O12" s="179"/>
-      <c r="P12" s="179"/>
-      <c r="Q12" s="179"/>
-      <c r="R12" s="172"/>
-      <c r="S12" s="173"/>
-      <c r="T12" s="177"/>
+      <c r="N12" s="176"/>
+      <c r="O12" s="176"/>
+      <c r="P12" s="176"/>
+      <c r="Q12" s="176"/>
+      <c r="R12" s="169"/>
+      <c r="S12" s="170"/>
+      <c r="T12" s="174"/>
     </row>
     <row r="13" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="158"/>
-      <c r="B13" s="159"/>
-      <c r="C13" s="161"/>
-      <c r="D13" s="181" t="s">
+      <c r="A13" s="155"/>
+      <c r="B13" s="156"/>
+      <c r="C13" s="158"/>
+      <c r="D13" s="178" t="s">
         <v>36</v>
       </c>
       <c r="E13" s="117" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="182" t="s">
+      <c r="F13" s="179" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="183"/>
-      <c r="H13" s="184" t="s">
+      <c r="G13" s="180"/>
+      <c r="H13" s="181" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="185"/>
-      <c r="J13" s="185"/>
-      <c r="K13" s="185"/>
-      <c r="L13" s="160" t="s">
+      <c r="I13" s="182"/>
+      <c r="J13" s="182"/>
+      <c r="K13" s="182"/>
+      <c r="L13" s="157" t="s">
         <v>41</v>
       </c>
-      <c r="M13" s="186" t="s">
+      <c r="M13" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="N13" s="187"/>
-      <c r="O13" s="188" t="s">
+      <c r="N13" s="184"/>
+      <c r="O13" s="185" t="s">
         <v>25</v>
       </c>
-      <c r="P13" s="188"/>
+      <c r="P13" s="185"/>
       <c r="Q13" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="R13" s="172"/>
-      <c r="S13" s="173"/>
-      <c r="T13" s="177"/>
+      <c r="R13" s="169"/>
+      <c r="S13" s="170"/>
+      <c r="T13" s="174"/>
     </row>
     <row r="14" spans="1:21" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="158"/>
-      <c r="B14" s="159"/>
-      <c r="C14" s="162"/>
-      <c r="D14" s="181"/>
+      <c r="A14" s="155"/>
+      <c r="B14" s="156"/>
+      <c r="C14" s="159"/>
+      <c r="D14" s="178"/>
       <c r="E14" s="117"/>
       <c r="F14" s="62" t="s">
         <v>28</v>
@@ -4036,8 +4020,8 @@
       <c r="K14" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="L14" s="162"/>
-      <c r="M14" s="189" t="s">
+      <c r="L14" s="159"/>
+      <c r="M14" s="186" t="s">
         <v>23</v>
       </c>
       <c r="N14" s="120"/>
@@ -4048,9 +4032,9 @@
       <c r="Q14" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="R14" s="174"/>
-      <c r="S14" s="175"/>
-      <c r="T14" s="177"/>
+      <c r="R14" s="171"/>
+      <c r="S14" s="172"/>
+      <c r="T14" s="174"/>
     </row>
     <row r="15" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="21">
@@ -4085,13 +4069,13 @@
       <c r="L15" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="M15" s="190"/>
-      <c r="N15" s="191"/>
-      <c r="O15" s="190"/>
-      <c r="P15" s="191"/>
+      <c r="M15" s="187"/>
+      <c r="N15" s="188"/>
+      <c r="O15" s="187"/>
+      <c r="P15" s="188"/>
       <c r="Q15" s="58"/>
-      <c r="R15" s="192"/>
-      <c r="S15" s="193"/>
+      <c r="R15" s="189"/>
+      <c r="S15" s="190"/>
       <c r="T15" s="64"/>
     </row>
     <row r="16" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4112,21 +4096,21 @@
       <c r="J16" s="46"/>
       <c r="K16" s="47"/>
       <c r="L16" s="42"/>
-      <c r="M16" s="194" t="s">
+      <c r="M16" s="191" t="s">
         <v>44</v>
       </c>
-      <c r="N16" s="195"/>
-      <c r="O16" s="196" t="s">
+      <c r="N16" s="192"/>
+      <c r="O16" s="193" t="s">
         <v>44</v>
       </c>
-      <c r="P16" s="197"/>
+      <c r="P16" s="194"/>
       <c r="Q16" s="58" t="s">
         <v>46</v>
       </c>
-      <c r="R16" s="192" t="s">
+      <c r="R16" s="189" t="s">
         <v>15</v>
       </c>
-      <c r="S16" s="193"/>
+      <c r="S16" s="190"/>
       <c r="T16" s="64" t="s">
         <v>15</v>
       </c>
@@ -4146,21 +4130,21 @@
       <c r="J17" s="46"/>
       <c r="K17" s="47"/>
       <c r="L17" s="42"/>
-      <c r="M17" s="194" t="s">
+      <c r="M17" s="191" t="s">
         <v>45</v>
       </c>
-      <c r="N17" s="195"/>
-      <c r="O17" s="196" t="s">
+      <c r="N17" s="192"/>
+      <c r="O17" s="193" t="s">
         <v>46</v>
       </c>
-      <c r="P17" s="197"/>
+      <c r="P17" s="194"/>
       <c r="Q17" s="74" t="s">
-        <v>54</v>
-      </c>
-      <c r="R17" s="198" t="s">
+        <v>53</v>
+      </c>
+      <c r="R17" s="195" t="s">
         <v>48</v>
       </c>
-      <c r="S17" s="199"/>
+      <c r="S17" s="196"/>
       <c r="T17" s="64" t="s">
         <v>46</v>
       </c>
@@ -4180,21 +4164,21 @@
       <c r="J18" s="46"/>
       <c r="K18" s="47"/>
       <c r="L18" s="42"/>
-      <c r="M18" s="194" t="s">
+      <c r="M18" s="191" t="s">
         <v>45</v>
       </c>
-      <c r="N18" s="195"/>
-      <c r="O18" s="196" t="s">
+      <c r="N18" s="192"/>
+      <c r="O18" s="193" t="s">
         <v>46</v>
       </c>
-      <c r="P18" s="197"/>
+      <c r="P18" s="194"/>
       <c r="Q18" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="R18" s="200" t="s">
+      <c r="R18" s="197" t="s">
         <v>47</v>
       </c>
-      <c r="S18" s="201"/>
+      <c r="S18" s="198"/>
       <c r="T18" s="64" t="s">
         <v>46</v>
       </c>
@@ -4214,13 +4198,13 @@
       <c r="J19" s="46"/>
       <c r="K19" s="47"/>
       <c r="L19" s="42"/>
-      <c r="M19" s="194"/>
-      <c r="N19" s="195"/>
-      <c r="O19" s="196"/>
-      <c r="P19" s="197"/>
+      <c r="M19" s="191"/>
+      <c r="N19" s="192"/>
+      <c r="O19" s="193"/>
+      <c r="P19" s="194"/>
       <c r="Q19" s="58"/>
-      <c r="R19" s="192"/>
-      <c r="S19" s="193"/>
+      <c r="R19" s="189"/>
+      <c r="S19" s="190"/>
       <c r="T19" s="64"/>
     </row>
     <row r="20" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4238,13 +4222,13 @@
       <c r="J20" s="46"/>
       <c r="K20" s="47"/>
       <c r="L20" s="42"/>
-      <c r="M20" s="194"/>
-      <c r="N20" s="195"/>
-      <c r="O20" s="196"/>
-      <c r="P20" s="197"/>
+      <c r="M20" s="191"/>
+      <c r="N20" s="192"/>
+      <c r="O20" s="193"/>
+      <c r="P20" s="194"/>
       <c r="Q20" s="58"/>
-      <c r="R20" s="192"/>
-      <c r="S20" s="193"/>
+      <c r="R20" s="189"/>
+      <c r="S20" s="190"/>
       <c r="T20" s="64"/>
     </row>
     <row r="21" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4262,13 +4246,13 @@
       <c r="J21" s="46"/>
       <c r="K21" s="47"/>
       <c r="L21" s="42"/>
-      <c r="M21" s="194"/>
-      <c r="N21" s="195"/>
-      <c r="O21" s="196"/>
-      <c r="P21" s="197"/>
+      <c r="M21" s="191"/>
+      <c r="N21" s="192"/>
+      <c r="O21" s="193"/>
+      <c r="P21" s="194"/>
       <c r="Q21" s="58"/>
-      <c r="R21" s="192"/>
-      <c r="S21" s="193"/>
+      <c r="R21" s="189"/>
+      <c r="S21" s="190"/>
       <c r="T21" s="64"/>
     </row>
     <row r="22" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4286,13 +4270,13 @@
       <c r="J22" s="46"/>
       <c r="K22" s="47"/>
       <c r="L22" s="42"/>
-      <c r="M22" s="194"/>
-      <c r="N22" s="195"/>
-      <c r="O22" s="196"/>
-      <c r="P22" s="197"/>
+      <c r="M22" s="191"/>
+      <c r="N22" s="192"/>
+      <c r="O22" s="193"/>
+      <c r="P22" s="194"/>
       <c r="Q22" s="58"/>
-      <c r="R22" s="192"/>
-      <c r="S22" s="193"/>
+      <c r="R22" s="189"/>
+      <c r="S22" s="190"/>
       <c r="T22" s="64"/>
     </row>
     <row r="23" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4310,13 +4294,13 @@
       <c r="J23" s="46"/>
       <c r="K23" s="47"/>
       <c r="L23" s="42"/>
-      <c r="M23" s="194"/>
-      <c r="N23" s="195"/>
-      <c r="O23" s="196"/>
-      <c r="P23" s="197"/>
+      <c r="M23" s="191"/>
+      <c r="N23" s="192"/>
+      <c r="O23" s="193"/>
+      <c r="P23" s="194"/>
       <c r="Q23" s="58"/>
-      <c r="R23" s="192"/>
-      <c r="S23" s="193"/>
+      <c r="R23" s="189"/>
+      <c r="S23" s="190"/>
       <c r="T23" s="64"/>
     </row>
     <row r="24" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4334,13 +4318,13 @@
       <c r="J24" s="46"/>
       <c r="K24" s="47"/>
       <c r="L24" s="42"/>
-      <c r="M24" s="194"/>
-      <c r="N24" s="195"/>
-      <c r="O24" s="196"/>
-      <c r="P24" s="197"/>
+      <c r="M24" s="191"/>
+      <c r="N24" s="192"/>
+      <c r="O24" s="193"/>
+      <c r="P24" s="194"/>
       <c r="Q24" s="58"/>
-      <c r="R24" s="192"/>
-      <c r="S24" s="193"/>
+      <c r="R24" s="189"/>
+      <c r="S24" s="190"/>
       <c r="T24" s="64"/>
     </row>
     <row r="25" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4358,13 +4342,13 @@
       <c r="J25" s="46"/>
       <c r="K25" s="47"/>
       <c r="L25" s="42"/>
-      <c r="M25" s="194"/>
-      <c r="N25" s="195"/>
-      <c r="O25" s="196"/>
-      <c r="P25" s="197"/>
+      <c r="M25" s="191"/>
+      <c r="N25" s="192"/>
+      <c r="O25" s="193"/>
+      <c r="P25" s="194"/>
       <c r="Q25" s="58"/>
-      <c r="R25" s="192"/>
-      <c r="S25" s="193"/>
+      <c r="R25" s="189"/>
+      <c r="S25" s="190"/>
       <c r="T25" s="64"/>
     </row>
     <row r="26" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4382,13 +4366,13 @@
       <c r="J26" s="46"/>
       <c r="K26" s="47"/>
       <c r="L26" s="42"/>
-      <c r="M26" s="194"/>
-      <c r="N26" s="195"/>
-      <c r="O26" s="196"/>
-      <c r="P26" s="197"/>
+      <c r="M26" s="191"/>
+      <c r="N26" s="192"/>
+      <c r="O26" s="193"/>
+      <c r="P26" s="194"/>
       <c r="Q26" s="58"/>
-      <c r="R26" s="192"/>
-      <c r="S26" s="193"/>
+      <c r="R26" s="189"/>
+      <c r="S26" s="190"/>
       <c r="T26" s="64"/>
     </row>
     <row r="27" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4406,13 +4390,13 @@
       <c r="J27" s="46"/>
       <c r="K27" s="47"/>
       <c r="L27" s="42"/>
-      <c r="M27" s="194"/>
-      <c r="N27" s="195"/>
-      <c r="O27" s="196"/>
-      <c r="P27" s="197"/>
+      <c r="M27" s="191"/>
+      <c r="N27" s="192"/>
+      <c r="O27" s="193"/>
+      <c r="P27" s="194"/>
       <c r="Q27" s="58"/>
-      <c r="R27" s="192"/>
-      <c r="S27" s="193"/>
+      <c r="R27" s="189"/>
+      <c r="S27" s="190"/>
       <c r="T27" s="64"/>
     </row>
     <row r="28" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4430,13 +4414,13 @@
       <c r="J28" s="46"/>
       <c r="K28" s="47"/>
       <c r="L28" s="42"/>
-      <c r="M28" s="194"/>
-      <c r="N28" s="195"/>
-      <c r="O28" s="196"/>
-      <c r="P28" s="197"/>
+      <c r="M28" s="191"/>
+      <c r="N28" s="192"/>
+      <c r="O28" s="193"/>
+      <c r="P28" s="194"/>
       <c r="Q28" s="59"/>
-      <c r="R28" s="192"/>
-      <c r="S28" s="193"/>
+      <c r="R28" s="189"/>
+      <c r="S28" s="190"/>
       <c r="T28" s="64"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4520,12 +4504,12 @@
       <c r="U32" s="2"/>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A33" s="202" t="s">
+      <c r="A33" s="199" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="202"/>
-      <c r="C33" s="202"/>
-      <c r="D33" s="202"/>
+      <c r="B33" s="199"/>
+      <c r="C33" s="199"/>
+      <c r="D33" s="199"/>
       <c r="E33" s="35"/>
       <c r="F33" s="35"/>
       <c r="G33" s="35"/>
@@ -4545,12 +4529,12 @@
       <c r="U33" s="2"/>
     </row>
     <row r="34" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="203" t="s">
+      <c r="A34" s="200" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="203"/>
-      <c r="C34" s="203"/>
-      <c r="D34" s="203"/>
+      <c r="B34" s="200"/>
+      <c r="C34" s="200"/>
+      <c r="D34" s="200"/>
       <c r="E34" s="36"/>
       <c r="F34" s="36"/>
       <c r="G34" s="36"/>

</xml_diff>

<commit_message>
fix(verificacion): preserve spacer row and refresh template
</commit_message>
<xml_diff>
--- a/app/templates/Template_Verificacion.xlsx
+++ b/app/templates/Template_Verificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A3CA2A-2E3A-400F-87EE-0EFDB107D714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA5BCF6-4A54-4C9E-81D1-736E25B6FA44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A76715E4-29FC-4532-A462-AEFC175FF6CC}"/>
   </bookViews>
@@ -608,7 +608,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="&quot;0&quot;0"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="29" x14ac:knownFonts="1">
     <font>
@@ -1526,59 +1526,23 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1593,44 +1557,209 @@
     <xf numFmtId="0" fontId="28" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1644,161 +1773,32 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2556,107 +2556,115 @@
       <c r="A1" s="65"/>
       <c r="B1" s="66"/>
       <c r="C1" s="67"/>
-      <c r="D1" s="137" t="s">
+      <c r="D1" s="126" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="137"/>
-      <c r="F1" s="137"/>
-      <c r="G1" s="137"/>
-      <c r="H1" s="137"/>
-      <c r="I1" s="137"/>
-      <c r="J1" s="137"/>
-      <c r="K1" s="137"/>
-      <c r="L1" s="137"/>
-      <c r="M1" s="137"/>
-      <c r="N1" s="137"/>
-      <c r="O1" s="137"/>
-      <c r="P1" s="137"/>
-      <c r="Q1" s="137"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="126"/>
+      <c r="J1" s="126"/>
+      <c r="K1" s="126"/>
+      <c r="L1" s="126"/>
+      <c r="M1" s="126"/>
+      <c r="N1" s="126"/>
+      <c r="O1" s="126"/>
+      <c r="P1" s="126"/>
+      <c r="Q1" s="126"/>
+      <c r="R1" s="126"/>
+      <c r="S1" s="126"/>
       <c r="T1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="U1" s="149" t="s">
+      <c r="U1" s="117" t="s">
         <v>16</v>
       </c>
-      <c r="V1" s="150"/>
+      <c r="V1" s="118"/>
     </row>
     <row r="2" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="68"/>
       <c r="B2" s="4"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="137"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="137"/>
-      <c r="H2" s="137"/>
-      <c r="I2" s="137"/>
-      <c r="J2" s="137"/>
-      <c r="K2" s="137"/>
-      <c r="L2" s="137"/>
-      <c r="M2" s="137"/>
-      <c r="N2" s="137"/>
-      <c r="O2" s="137"/>
-      <c r="P2" s="137"/>
-      <c r="Q2" s="137"/>
+      <c r="D2" s="126"/>
+      <c r="E2" s="126"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="126"/>
+      <c r="H2" s="126"/>
+      <c r="I2" s="126"/>
+      <c r="J2" s="126"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="126"/>
+      <c r="M2" s="126"/>
+      <c r="N2" s="126"/>
+      <c r="O2" s="126"/>
+      <c r="P2" s="126"/>
+      <c r="Q2" s="126"/>
+      <c r="R2" s="126"/>
+      <c r="S2" s="126"/>
       <c r="T2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="U2" s="201">
+      <c r="U2" s="119">
         <v>3</v>
       </c>
-      <c r="V2" s="202"/>
+      <c r="V2" s="120"/>
     </row>
     <row r="3" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="68"/>
       <c r="B3" s="4"/>
       <c r="C3" s="69"/>
-      <c r="D3" s="137"/>
-      <c r="E3" s="137"/>
-      <c r="F3" s="137"/>
-      <c r="G3" s="137"/>
-      <c r="H3" s="137"/>
-      <c r="I3" s="137"/>
-      <c r="J3" s="137"/>
-      <c r="K3" s="137"/>
-      <c r="L3" s="137"/>
-      <c r="M3" s="137"/>
-      <c r="N3" s="137"/>
-      <c r="O3" s="137"/>
-      <c r="P3" s="137"/>
-      <c r="Q3" s="137"/>
+      <c r="D3" s="126"/>
+      <c r="E3" s="126"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="126"/>
+      <c r="H3" s="126"/>
+      <c r="I3" s="126"/>
+      <c r="J3" s="126"/>
+      <c r="K3" s="126"/>
+      <c r="L3" s="126"/>
+      <c r="M3" s="126"/>
+      <c r="N3" s="126"/>
+      <c r="O3" s="126"/>
+      <c r="P3" s="126"/>
+      <c r="Q3" s="126"/>
+      <c r="R3" s="126"/>
+      <c r="S3" s="126"/>
       <c r="T3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="U3" s="203">
+      <c r="U3" s="121">
         <v>46104</v>
       </c>
-      <c r="V3" s="204"/>
+      <c r="V3" s="122"/>
     </row>
     <row r="4" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="70"/>
       <c r="B4" s="71"/>
       <c r="C4" s="72"/>
-      <c r="D4" s="137"/>
-      <c r="E4" s="137"/>
-      <c r="F4" s="137"/>
-      <c r="G4" s="137"/>
-      <c r="H4" s="137"/>
-      <c r="I4" s="137"/>
-      <c r="J4" s="137"/>
-      <c r="K4" s="137"/>
-      <c r="L4" s="137"/>
-      <c r="M4" s="137"/>
-      <c r="N4" s="137"/>
-      <c r="O4" s="137"/>
-      <c r="P4" s="137"/>
-      <c r="Q4" s="137"/>
+      <c r="D4" s="126"/>
+      <c r="E4" s="126"/>
+      <c r="F4" s="126"/>
+      <c r="G4" s="126"/>
+      <c r="H4" s="126"/>
+      <c r="I4" s="126"/>
+      <c r="J4" s="126"/>
+      <c r="K4" s="126"/>
+      <c r="L4" s="126"/>
+      <c r="M4" s="126"/>
+      <c r="N4" s="126"/>
+      <c r="O4" s="126"/>
+      <c r="P4" s="126"/>
+      <c r="Q4" s="126"/>
+      <c r="R4" s="126"/>
+      <c r="S4" s="126"/>
       <c r="T4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="U4" s="149" t="s">
+      <c r="U4" s="117" t="s">
         <v>4</v>
       </c>
-      <c r="V4" s="150"/>
+      <c r="V4" s="118"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
@@ -2682,20 +2690,20 @@
       <c r="B6" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="136"/>
-      <c r="D6" s="136"/>
-      <c r="E6" s="136"/>
-      <c r="F6" s="136"/>
-      <c r="G6" s="136"/>
-      <c r="H6" s="136"/>
-      <c r="I6" s="136"/>
-      <c r="J6" s="135" t="s">
+      <c r="C6" s="125"/>
+      <c r="D6" s="125"/>
+      <c r="E6" s="125"/>
+      <c r="F6" s="125"/>
+      <c r="G6" s="125"/>
+      <c r="H6" s="125"/>
+      <c r="I6" s="125"/>
+      <c r="J6" s="124" t="s">
         <v>52</v>
       </c>
-      <c r="K6" s="135"/>
-      <c r="L6" s="135"/>
-      <c r="M6" s="134"/>
-      <c r="N6" s="134"/>
+      <c r="K6" s="124"/>
+      <c r="L6" s="124"/>
+      <c r="M6" s="123"/>
+      <c r="N6" s="123"/>
       <c r="P6" s="76" t="s">
         <v>98</v>
       </c>
@@ -2706,68 +2714,68 @@
       <c r="A7" s="23"/>
       <c r="B7" s="23"/>
       <c r="C7" s="23"/>
-      <c r="D7" s="125"/>
-      <c r="E7" s="125"/>
-      <c r="F7" s="125"/>
-      <c r="G7" s="125"/>
-      <c r="H7" s="126"/>
-      <c r="I7" s="126"/>
-      <c r="J7" s="126"/>
-      <c r="K7" s="126"/>
-      <c r="L7" s="126"/>
+      <c r="D7" s="127"/>
+      <c r="E7" s="127"/>
+      <c r="F7" s="127"/>
+      <c r="G7" s="127"/>
+      <c r="H7" s="128"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="128"/>
+      <c r="K7" s="128"/>
+      <c r="L7" s="128"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
     </row>
     <row r="8" spans="1:22" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="128" t="s">
+      <c r="A8" s="130" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="128" t="s">
+      <c r="B8" s="130" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="130" t="s">
+      <c r="C8" s="132" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="118" t="s">
+      <c r="D8" s="137" t="s">
         <v>88</v>
       </c>
-      <c r="E8" s="118"/>
-      <c r="F8" s="118"/>
-      <c r="G8" s="118"/>
-      <c r="H8" s="119" t="s">
+      <c r="E8" s="137"/>
+      <c r="F8" s="137"/>
+      <c r="G8" s="137"/>
+      <c r="H8" s="138" t="s">
         <v>67</v>
       </c>
-      <c r="I8" s="120"/>
-      <c r="J8" s="120"/>
-      <c r="K8" s="120"/>
-      <c r="L8" s="121"/>
-      <c r="M8" s="118" t="s">
+      <c r="I8" s="139"/>
+      <c r="J8" s="139"/>
+      <c r="K8" s="139"/>
+      <c r="L8" s="140"/>
+      <c r="M8" s="137" t="s">
         <v>12</v>
       </c>
-      <c r="N8" s="118"/>
-      <c r="O8" s="118"/>
-      <c r="P8" s="132" t="s">
+      <c r="N8" s="137"/>
+      <c r="O8" s="137"/>
+      <c r="P8" s="134" t="s">
         <v>77</v>
       </c>
-      <c r="Q8" s="132" t="s">
+      <c r="Q8" s="134" t="s">
         <v>79</v>
       </c>
-      <c r="R8" s="122" t="s">
+      <c r="R8" s="141" t="s">
         <v>81</v>
       </c>
-      <c r="S8" s="123"/>
-      <c r="T8" s="124"/>
-      <c r="U8" s="117" t="s">
+      <c r="S8" s="142"/>
+      <c r="T8" s="143"/>
+      <c r="U8" s="136" t="s">
         <v>82</v>
       </c>
-      <c r="V8" s="117"/>
+      <c r="V8" s="136"/>
     </row>
     <row r="9" spans="1:22" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="129"/>
-      <c r="B9" s="129"/>
-      <c r="C9" s="131"/>
+      <c r="A9" s="131"/>
+      <c r="B9" s="131"/>
+      <c r="C9" s="133"/>
       <c r="D9" s="87" t="s">
         <v>36</v>
       </c>
@@ -2804,8 +2812,8 @@
       <c r="O9" s="86" t="s">
         <v>96</v>
       </c>
-      <c r="P9" s="133"/>
-      <c r="Q9" s="133"/>
+      <c r="P9" s="135"/>
+      <c r="Q9" s="135"/>
       <c r="R9" s="87" t="s">
         <v>55</v>
       </c>
@@ -2815,8 +2823,8 @@
       <c r="T9" s="87" t="s">
         <v>57</v>
       </c>
-      <c r="U9" s="117"/>
-      <c r="V9" s="117"/>
+      <c r="U9" s="136"/>
+      <c r="V9" s="136"/>
     </row>
     <row r="10" spans="1:22" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="21"/>
@@ -3088,25 +3096,25 @@
       <c r="R20" s="2"/>
     </row>
     <row r="21" spans="1:22" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="127" t="s">
+      <c r="A21" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="127"/>
-      <c r="C21" s="127"/>
-      <c r="D21" s="127"/>
-      <c r="E21" s="127"/>
-      <c r="F21" s="127"/>
-      <c r="G21" s="127"/>
-      <c r="H21" s="127"/>
-      <c r="I21" s="127"/>
-      <c r="J21" s="127"/>
-      <c r="K21" s="127"/>
-      <c r="L21" s="127"/>
-      <c r="M21" s="127"/>
-      <c r="N21" s="127"/>
-      <c r="O21" s="127"/>
-      <c r="P21" s="127"/>
-      <c r="Q21" s="127"/>
+      <c r="B21" s="129"/>
+      <c r="C21" s="129"/>
+      <c r="D21" s="129"/>
+      <c r="E21" s="129"/>
+      <c r="F21" s="129"/>
+      <c r="G21" s="129"/>
+      <c r="H21" s="129"/>
+      <c r="I21" s="129"/>
+      <c r="J21" s="129"/>
+      <c r="K21" s="129"/>
+      <c r="L21" s="129"/>
+      <c r="M21" s="129"/>
+      <c r="N21" s="129"/>
+      <c r="O21" s="129"/>
+      <c r="P21" s="129"/>
+      <c r="Q21" s="129"/>
       <c r="R21" s="2"/>
     </row>
     <row r="22" spans="1:22" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3475,27 +3483,27 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="U2:V2"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="U4:V4"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="D1:Q4"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="H7:L7"/>
+    <mergeCell ref="U8:V9"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="M8:O8"/>
+    <mergeCell ref="H8:L8"/>
+    <mergeCell ref="R8:T8"/>
     <mergeCell ref="A21:Q21"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="P8:P9"/>
     <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="U8:V9"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="H8:L8"/>
-    <mergeCell ref="R8:T8"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="H7:L7"/>
+    <mergeCell ref="D1:S4"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="U2:V2"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="U4:V4"/>
+    <mergeCell ref="M6:N6"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.19685039370078741" header="0" footer="0"/>
@@ -3560,34 +3568,34 @@
       </c>
     </row>
     <row r="7" spans="2:5" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="138" t="s">
+      <c r="B7" s="144" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="139" t="s">
+      <c r="C7" s="145" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="98" t="s">
         <v>69</v>
       </c>
-      <c r="E7" s="138" t="s">
+      <c r="E7" s="144" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="138"/>
-      <c r="C8" s="139"/>
+      <c r="B8" s="144"/>
+      <c r="C8" s="145"/>
       <c r="D8" s="98" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="138"/>
+      <c r="E8" s="144"/>
     </row>
     <row r="9" spans="2:5" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="138"/>
-      <c r="C9" s="139"/>
+      <c r="B9" s="144"/>
+      <c r="C9" s="145"/>
       <c r="D9" s="98" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="138"/>
+      <c r="E9" s="144"/>
     </row>
     <row r="11" spans="2:5" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="99" t="s">
@@ -3649,110 +3657,110 @@
       <c r="A1" s="65"/>
       <c r="B1" s="66"/>
       <c r="C1" s="67"/>
-      <c r="D1" s="140" t="s">
+      <c r="D1" s="196" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="141"/>
-      <c r="F1" s="141"/>
-      <c r="G1" s="141"/>
-      <c r="H1" s="141"/>
-      <c r="I1" s="141"/>
-      <c r="J1" s="141"/>
-      <c r="K1" s="141"/>
-      <c r="L1" s="141"/>
-      <c r="M1" s="141"/>
-      <c r="N1" s="141"/>
-      <c r="O1" s="141"/>
-      <c r="P1" s="141"/>
-      <c r="Q1" s="142"/>
+      <c r="E1" s="197"/>
+      <c r="F1" s="197"/>
+      <c r="G1" s="197"/>
+      <c r="H1" s="197"/>
+      <c r="I1" s="197"/>
+      <c r="J1" s="197"/>
+      <c r="K1" s="197"/>
+      <c r="L1" s="197"/>
+      <c r="M1" s="197"/>
+      <c r="N1" s="197"/>
+      <c r="O1" s="197"/>
+      <c r="P1" s="197"/>
+      <c r="Q1" s="198"/>
       <c r="R1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="S1" s="149" t="s">
+      <c r="S1" s="117" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="150"/>
+      <c r="T1" s="118"/>
       <c r="U1" s="1"/>
     </row>
     <row r="2" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="68"/>
       <c r="B2" s="4"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="143"/>
-      <c r="E2" s="144"/>
-      <c r="F2" s="144"/>
-      <c r="G2" s="144"/>
-      <c r="H2" s="144"/>
-      <c r="I2" s="144"/>
-      <c r="J2" s="144"/>
-      <c r="K2" s="144"/>
-      <c r="L2" s="144"/>
-      <c r="M2" s="144"/>
-      <c r="N2" s="144"/>
-      <c r="O2" s="144"/>
-      <c r="P2" s="144"/>
-      <c r="Q2" s="145"/>
+      <c r="D2" s="199"/>
+      <c r="E2" s="200"/>
+      <c r="F2" s="200"/>
+      <c r="G2" s="200"/>
+      <c r="H2" s="200"/>
+      <c r="I2" s="200"/>
+      <c r="J2" s="200"/>
+      <c r="K2" s="200"/>
+      <c r="L2" s="200"/>
+      <c r="M2" s="200"/>
+      <c r="N2" s="200"/>
+      <c r="O2" s="200"/>
+      <c r="P2" s="200"/>
+      <c r="Q2" s="201"/>
       <c r="R2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="S2" s="149">
+      <c r="S2" s="117">
         <v>1</v>
       </c>
-      <c r="T2" s="150"/>
+      <c r="T2" s="118"/>
       <c r="U2" s="1"/>
     </row>
     <row r="3" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="68"/>
       <c r="B3" s="4"/>
       <c r="C3" s="69"/>
-      <c r="D3" s="143"/>
-      <c r="E3" s="144"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="144"/>
-      <c r="H3" s="144"/>
-      <c r="I3" s="144"/>
-      <c r="J3" s="144"/>
-      <c r="K3" s="144"/>
-      <c r="L3" s="144"/>
-      <c r="M3" s="144"/>
-      <c r="N3" s="144"/>
-      <c r="O3" s="144"/>
-      <c r="P3" s="144"/>
-      <c r="Q3" s="145"/>
+      <c r="D3" s="199"/>
+      <c r="E3" s="200"/>
+      <c r="F3" s="200"/>
+      <c r="G3" s="200"/>
+      <c r="H3" s="200"/>
+      <c r="I3" s="200"/>
+      <c r="J3" s="200"/>
+      <c r="K3" s="200"/>
+      <c r="L3" s="200"/>
+      <c r="M3" s="200"/>
+      <c r="N3" s="200"/>
+      <c r="O3" s="200"/>
+      <c r="P3" s="200"/>
+      <c r="Q3" s="201"/>
       <c r="R3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="S3" s="149">
+      <c r="S3" s="117">
         <v>45232</v>
       </c>
-      <c r="T3" s="150"/>
+      <c r="T3" s="118"/>
       <c r="U3" s="1"/>
     </row>
     <row r="4" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="70"/>
       <c r="B4" s="71"/>
       <c r="C4" s="72"/>
-      <c r="D4" s="146"/>
-      <c r="E4" s="147"/>
-      <c r="F4" s="147"/>
-      <c r="G4" s="147"/>
-      <c r="H4" s="147"/>
-      <c r="I4" s="147"/>
-      <c r="J4" s="147"/>
-      <c r="K4" s="147"/>
-      <c r="L4" s="147"/>
-      <c r="M4" s="147"/>
-      <c r="N4" s="147"/>
-      <c r="O4" s="147"/>
-      <c r="P4" s="147"/>
-      <c r="Q4" s="148"/>
+      <c r="D4" s="202"/>
+      <c r="E4" s="203"/>
+      <c r="F4" s="203"/>
+      <c r="G4" s="203"/>
+      <c r="H4" s="203"/>
+      <c r="I4" s="203"/>
+      <c r="J4" s="203"/>
+      <c r="K4" s="203"/>
+      <c r="L4" s="203"/>
+      <c r="M4" s="203"/>
+      <c r="N4" s="203"/>
+      <c r="O4" s="203"/>
+      <c r="P4" s="203"/>
+      <c r="Q4" s="204"/>
       <c r="R4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="S4" s="149" t="s">
+      <c r="S4" s="117" t="s">
         <v>4</v>
       </c>
-      <c r="T4" s="150"/>
+      <c r="T4" s="118"/>
       <c r="U4" s="1"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -3785,16 +3793,16 @@
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
       <c r="D6" s="27"/>
-      <c r="E6" s="151"/>
-      <c r="F6" s="151"/>
+      <c r="E6" s="192"/>
+      <c r="F6" s="192"/>
       <c r="G6" s="28"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="152" t="s">
+      <c r="J6" s="193" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="152"/>
-      <c r="L6" s="152"/>
+      <c r="K6" s="193"/>
+      <c r="L6" s="193"/>
       <c r="M6" s="33"/>
       <c r="N6" s="52"/>
       <c r="O6" s="33"/>
@@ -3812,11 +3820,11 @@
       <c r="D7" s="18"/>
       <c r="E7" s="9"/>
       <c r="F7" s="10"/>
-      <c r="G7" s="153"/>
-      <c r="H7" s="153"/>
-      <c r="I7" s="153"/>
-      <c r="J7" s="153"/>
-      <c r="K7" s="153"/>
+      <c r="G7" s="194"/>
+      <c r="H7" s="194"/>
+      <c r="I7" s="194"/>
+      <c r="J7" s="194"/>
+      <c r="K7" s="194"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -3830,10 +3838,10 @@
       <c r="B8" s="23"/>
       <c r="C8" s="23"/>
       <c r="D8" s="29"/>
-      <c r="E8" s="154"/>
-      <c r="F8" s="154"/>
-      <c r="G8" s="154"/>
-      <c r="H8" s="154"/>
+      <c r="E8" s="195"/>
+      <c r="F8" s="195"/>
+      <c r="G8" s="195"/>
+      <c r="H8" s="195"/>
       <c r="I8" s="34"/>
       <c r="J8" s="34"/>
       <c r="K8" s="34"/>
@@ -3853,10 +3861,10 @@
       <c r="B9" s="23"/>
       <c r="C9" s="23"/>
       <c r="D9" s="29"/>
-      <c r="E9" s="154"/>
-      <c r="F9" s="154"/>
-      <c r="G9" s="154"/>
-      <c r="H9" s="154"/>
+      <c r="E9" s="195"/>
+      <c r="F9" s="195"/>
+      <c r="G9" s="195"/>
+      <c r="H9" s="195"/>
       <c r="I9" s="34"/>
       <c r="J9" s="34"/>
       <c r="K9" s="34"/>
@@ -3872,19 +3880,19 @@
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>
-      <c r="D10" s="125" t="s">
+      <c r="D10" s="127" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="125"/>
-      <c r="F10" s="125"/>
-      <c r="G10" s="125"/>
-      <c r="H10" s="126" t="s">
+      <c r="E10" s="127"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="127"/>
+      <c r="H10" s="128" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="126"/>
-      <c r="J10" s="126"/>
-      <c r="K10" s="126"/>
-      <c r="L10" s="126"/>
+      <c r="I10" s="128"/>
+      <c r="J10" s="128"/>
+      <c r="K10" s="128"/>
+      <c r="L10" s="128"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
@@ -3892,116 +3900,116 @@
       <c r="U10" s="1"/>
     </row>
     <row r="11" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="155" t="s">
+      <c r="A11" s="184" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="156" t="s">
+      <c r="B11" s="185" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="157" t="s">
+      <c r="C11" s="178" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="160" t="s">
+      <c r="D11" s="187" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="161"/>
-      <c r="F11" s="161"/>
-      <c r="G11" s="162"/>
-      <c r="H11" s="163" t="s">
+      <c r="E11" s="188"/>
+      <c r="F11" s="188"/>
+      <c r="G11" s="189"/>
+      <c r="H11" s="190" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="164"/>
-      <c r="J11" s="164"/>
-      <c r="K11" s="164"/>
-      <c r="L11" s="164"/>
-      <c r="M11" s="165" t="s">
+      <c r="I11" s="191"/>
+      <c r="J11" s="191"/>
+      <c r="K11" s="191"/>
+      <c r="L11" s="191"/>
+      <c r="M11" s="160" t="s">
         <v>18</v>
       </c>
-      <c r="N11" s="166"/>
-      <c r="O11" s="166"/>
-      <c r="P11" s="166"/>
-      <c r="Q11" s="166"/>
-      <c r="R11" s="167" t="s">
+      <c r="N11" s="161"/>
+      <c r="O11" s="161"/>
+      <c r="P11" s="161"/>
+      <c r="Q11" s="161"/>
+      <c r="R11" s="162" t="s">
         <v>34</v>
       </c>
-      <c r="S11" s="168"/>
-      <c r="T11" s="173" t="s">
+      <c r="S11" s="163"/>
+      <c r="T11" s="168" t="s">
         <v>33</v>
       </c>
       <c r="U11" s="1"/>
     </row>
     <row r="12" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="155"/>
-      <c r="B12" s="156"/>
-      <c r="C12" s="158"/>
-      <c r="D12" s="175" t="s">
+      <c r="A12" s="184"/>
+      <c r="B12" s="185"/>
+      <c r="C12" s="186"/>
+      <c r="D12" s="170" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="176"/>
-      <c r="F12" s="176"/>
-      <c r="G12" s="177"/>
-      <c r="H12" s="175" t="s">
+      <c r="E12" s="171"/>
+      <c r="F12" s="171"/>
+      <c r="G12" s="172"/>
+      <c r="H12" s="170" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="176"/>
-      <c r="J12" s="176"/>
-      <c r="K12" s="176"/>
-      <c r="L12" s="177"/>
-      <c r="M12" s="175" t="s">
+      <c r="I12" s="171"/>
+      <c r="J12" s="171"/>
+      <c r="K12" s="171"/>
+      <c r="L12" s="172"/>
+      <c r="M12" s="170" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="176"/>
-      <c r="O12" s="176"/>
-      <c r="P12" s="176"/>
-      <c r="Q12" s="176"/>
-      <c r="R12" s="169"/>
-      <c r="S12" s="170"/>
-      <c r="T12" s="174"/>
+      <c r="N12" s="171"/>
+      <c r="O12" s="171"/>
+      <c r="P12" s="171"/>
+      <c r="Q12" s="171"/>
+      <c r="R12" s="164"/>
+      <c r="S12" s="165"/>
+      <c r="T12" s="169"/>
     </row>
     <row r="13" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="155"/>
-      <c r="B13" s="156"/>
-      <c r="C13" s="158"/>
-      <c r="D13" s="178" t="s">
+      <c r="A13" s="184"/>
+      <c r="B13" s="185"/>
+      <c r="C13" s="186"/>
+      <c r="D13" s="173" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="117" t="s">
+      <c r="E13" s="136" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="179" t="s">
+      <c r="F13" s="174" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="180"/>
-      <c r="H13" s="181" t="s">
+      <c r="G13" s="175"/>
+      <c r="H13" s="176" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="182"/>
-      <c r="J13" s="182"/>
-      <c r="K13" s="182"/>
-      <c r="L13" s="157" t="s">
+      <c r="I13" s="177"/>
+      <c r="J13" s="177"/>
+      <c r="K13" s="177"/>
+      <c r="L13" s="178" t="s">
         <v>41</v>
       </c>
-      <c r="M13" s="183" t="s">
+      <c r="M13" s="180" t="s">
         <v>24</v>
       </c>
-      <c r="N13" s="184"/>
-      <c r="O13" s="185" t="s">
+      <c r="N13" s="181"/>
+      <c r="O13" s="182" t="s">
         <v>25</v>
       </c>
-      <c r="P13" s="185"/>
+      <c r="P13" s="182"/>
       <c r="Q13" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="R13" s="169"/>
-      <c r="S13" s="170"/>
-      <c r="T13" s="174"/>
+      <c r="R13" s="164"/>
+      <c r="S13" s="165"/>
+      <c r="T13" s="169"/>
     </row>
     <row r="14" spans="1:21" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="155"/>
-      <c r="B14" s="156"/>
-      <c r="C14" s="159"/>
-      <c r="D14" s="178"/>
-      <c r="E14" s="117"/>
+      <c r="A14" s="184"/>
+      <c r="B14" s="185"/>
+      <c r="C14" s="179"/>
+      <c r="D14" s="173"/>
+      <c r="E14" s="136"/>
       <c r="F14" s="62" t="s">
         <v>28</v>
       </c>
@@ -4020,21 +4028,21 @@
       <c r="K14" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="L14" s="159"/>
-      <c r="M14" s="186" t="s">
+      <c r="L14" s="179"/>
+      <c r="M14" s="183" t="s">
         <v>23</v>
       </c>
-      <c r="N14" s="120"/>
-      <c r="O14" s="119" t="s">
+      <c r="N14" s="139"/>
+      <c r="O14" s="138" t="s">
         <v>23</v>
       </c>
-      <c r="P14" s="121"/>
+      <c r="P14" s="140"/>
       <c r="Q14" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="R14" s="171"/>
-      <c r="S14" s="172"/>
-      <c r="T14" s="174"/>
+      <c r="R14" s="166"/>
+      <c r="S14" s="167"/>
+      <c r="T14" s="169"/>
     </row>
     <row r="15" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="21">
@@ -4069,13 +4077,13 @@
       <c r="L15" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="M15" s="187"/>
-      <c r="N15" s="188"/>
-      <c r="O15" s="187"/>
-      <c r="P15" s="188"/>
+      <c r="M15" s="158"/>
+      <c r="N15" s="159"/>
+      <c r="O15" s="158"/>
+      <c r="P15" s="159"/>
       <c r="Q15" s="58"/>
-      <c r="R15" s="189"/>
-      <c r="S15" s="190"/>
+      <c r="R15" s="152"/>
+      <c r="S15" s="153"/>
       <c r="T15" s="64"/>
     </row>
     <row r="16" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4096,21 +4104,21 @@
       <c r="J16" s="46"/>
       <c r="K16" s="47"/>
       <c r="L16" s="42"/>
-      <c r="M16" s="191" t="s">
+      <c r="M16" s="148" t="s">
         <v>44</v>
       </c>
-      <c r="N16" s="192"/>
-      <c r="O16" s="193" t="s">
+      <c r="N16" s="149"/>
+      <c r="O16" s="150" t="s">
         <v>44</v>
       </c>
-      <c r="P16" s="194"/>
+      <c r="P16" s="151"/>
       <c r="Q16" s="58" t="s">
         <v>46</v>
       </c>
-      <c r="R16" s="189" t="s">
+      <c r="R16" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="S16" s="190"/>
+      <c r="S16" s="153"/>
       <c r="T16" s="64" t="s">
         <v>15</v>
       </c>
@@ -4130,21 +4138,21 @@
       <c r="J17" s="46"/>
       <c r="K17" s="47"/>
       <c r="L17" s="42"/>
-      <c r="M17" s="191" t="s">
+      <c r="M17" s="148" t="s">
         <v>45</v>
       </c>
-      <c r="N17" s="192"/>
-      <c r="O17" s="193" t="s">
+      <c r="N17" s="149"/>
+      <c r="O17" s="150" t="s">
         <v>46</v>
       </c>
-      <c r="P17" s="194"/>
+      <c r="P17" s="151"/>
       <c r="Q17" s="74" t="s">
         <v>53</v>
       </c>
-      <c r="R17" s="195" t="s">
+      <c r="R17" s="154" t="s">
         <v>48</v>
       </c>
-      <c r="S17" s="196"/>
+      <c r="S17" s="155"/>
       <c r="T17" s="64" t="s">
         <v>46</v>
       </c>
@@ -4164,21 +4172,21 @@
       <c r="J18" s="46"/>
       <c r="K18" s="47"/>
       <c r="L18" s="42"/>
-      <c r="M18" s="191" t="s">
+      <c r="M18" s="148" t="s">
         <v>45</v>
       </c>
-      <c r="N18" s="192"/>
-      <c r="O18" s="193" t="s">
+      <c r="N18" s="149"/>
+      <c r="O18" s="150" t="s">
         <v>46</v>
       </c>
-      <c r="P18" s="194"/>
+      <c r="P18" s="151"/>
       <c r="Q18" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="R18" s="197" t="s">
+      <c r="R18" s="156" t="s">
         <v>47</v>
       </c>
-      <c r="S18" s="198"/>
+      <c r="S18" s="157"/>
       <c r="T18" s="64" t="s">
         <v>46</v>
       </c>
@@ -4198,13 +4206,13 @@
       <c r="J19" s="46"/>
       <c r="K19" s="47"/>
       <c r="L19" s="42"/>
-      <c r="M19" s="191"/>
-      <c r="N19" s="192"/>
-      <c r="O19" s="193"/>
-      <c r="P19" s="194"/>
+      <c r="M19" s="148"/>
+      <c r="N19" s="149"/>
+      <c r="O19" s="150"/>
+      <c r="P19" s="151"/>
       <c r="Q19" s="58"/>
-      <c r="R19" s="189"/>
-      <c r="S19" s="190"/>
+      <c r="R19" s="152"/>
+      <c r="S19" s="153"/>
       <c r="T19" s="64"/>
     </row>
     <row r="20" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4222,13 +4230,13 @@
       <c r="J20" s="46"/>
       <c r="K20" s="47"/>
       <c r="L20" s="42"/>
-      <c r="M20" s="191"/>
-      <c r="N20" s="192"/>
-      <c r="O20" s="193"/>
-      <c r="P20" s="194"/>
+      <c r="M20" s="148"/>
+      <c r="N20" s="149"/>
+      <c r="O20" s="150"/>
+      <c r="P20" s="151"/>
       <c r="Q20" s="58"/>
-      <c r="R20" s="189"/>
-      <c r="S20" s="190"/>
+      <c r="R20" s="152"/>
+      <c r="S20" s="153"/>
       <c r="T20" s="64"/>
     </row>
     <row r="21" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4246,13 +4254,13 @@
       <c r="J21" s="46"/>
       <c r="K21" s="47"/>
       <c r="L21" s="42"/>
-      <c r="M21" s="191"/>
-      <c r="N21" s="192"/>
-      <c r="O21" s="193"/>
-      <c r="P21" s="194"/>
+      <c r="M21" s="148"/>
+      <c r="N21" s="149"/>
+      <c r="O21" s="150"/>
+      <c r="P21" s="151"/>
       <c r="Q21" s="58"/>
-      <c r="R21" s="189"/>
-      <c r="S21" s="190"/>
+      <c r="R21" s="152"/>
+      <c r="S21" s="153"/>
       <c r="T21" s="64"/>
     </row>
     <row r="22" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4270,13 +4278,13 @@
       <c r="J22" s="46"/>
       <c r="K22" s="47"/>
       <c r="L22" s="42"/>
-      <c r="M22" s="191"/>
-      <c r="N22" s="192"/>
-      <c r="O22" s="193"/>
-      <c r="P22" s="194"/>
+      <c r="M22" s="148"/>
+      <c r="N22" s="149"/>
+      <c r="O22" s="150"/>
+      <c r="P22" s="151"/>
       <c r="Q22" s="58"/>
-      <c r="R22" s="189"/>
-      <c r="S22" s="190"/>
+      <c r="R22" s="152"/>
+      <c r="S22" s="153"/>
       <c r="T22" s="64"/>
     </row>
     <row r="23" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4294,13 +4302,13 @@
       <c r="J23" s="46"/>
       <c r="K23" s="47"/>
       <c r="L23" s="42"/>
-      <c r="M23" s="191"/>
-      <c r="N23" s="192"/>
-      <c r="O23" s="193"/>
-      <c r="P23" s="194"/>
+      <c r="M23" s="148"/>
+      <c r="N23" s="149"/>
+      <c r="O23" s="150"/>
+      <c r="P23" s="151"/>
       <c r="Q23" s="58"/>
-      <c r="R23" s="189"/>
-      <c r="S23" s="190"/>
+      <c r="R23" s="152"/>
+      <c r="S23" s="153"/>
       <c r="T23" s="64"/>
     </row>
     <row r="24" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4318,13 +4326,13 @@
       <c r="J24" s="46"/>
       <c r="K24" s="47"/>
       <c r="L24" s="42"/>
-      <c r="M24" s="191"/>
-      <c r="N24" s="192"/>
-      <c r="O24" s="193"/>
-      <c r="P24" s="194"/>
+      <c r="M24" s="148"/>
+      <c r="N24" s="149"/>
+      <c r="O24" s="150"/>
+      <c r="P24" s="151"/>
       <c r="Q24" s="58"/>
-      <c r="R24" s="189"/>
-      <c r="S24" s="190"/>
+      <c r="R24" s="152"/>
+      <c r="S24" s="153"/>
       <c r="T24" s="64"/>
     </row>
     <row r="25" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4342,13 +4350,13 @@
       <c r="J25" s="46"/>
       <c r="K25" s="47"/>
       <c r="L25" s="42"/>
-      <c r="M25" s="191"/>
-      <c r="N25" s="192"/>
-      <c r="O25" s="193"/>
-      <c r="P25" s="194"/>
+      <c r="M25" s="148"/>
+      <c r="N25" s="149"/>
+      <c r="O25" s="150"/>
+      <c r="P25" s="151"/>
       <c r="Q25" s="58"/>
-      <c r="R25" s="189"/>
-      <c r="S25" s="190"/>
+      <c r="R25" s="152"/>
+      <c r="S25" s="153"/>
       <c r="T25" s="64"/>
     </row>
     <row r="26" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4366,13 +4374,13 @@
       <c r="J26" s="46"/>
       <c r="K26" s="47"/>
       <c r="L26" s="42"/>
-      <c r="M26" s="191"/>
-      <c r="N26" s="192"/>
-      <c r="O26" s="193"/>
-      <c r="P26" s="194"/>
+      <c r="M26" s="148"/>
+      <c r="N26" s="149"/>
+      <c r="O26" s="150"/>
+      <c r="P26" s="151"/>
       <c r="Q26" s="58"/>
-      <c r="R26" s="189"/>
-      <c r="S26" s="190"/>
+      <c r="R26" s="152"/>
+      <c r="S26" s="153"/>
       <c r="T26" s="64"/>
     </row>
     <row r="27" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4390,13 +4398,13 @@
       <c r="J27" s="46"/>
       <c r="K27" s="47"/>
       <c r="L27" s="42"/>
-      <c r="M27" s="191"/>
-      <c r="N27" s="192"/>
-      <c r="O27" s="193"/>
-      <c r="P27" s="194"/>
+      <c r="M27" s="148"/>
+      <c r="N27" s="149"/>
+      <c r="O27" s="150"/>
+      <c r="P27" s="151"/>
       <c r="Q27" s="58"/>
-      <c r="R27" s="189"/>
-      <c r="S27" s="190"/>
+      <c r="R27" s="152"/>
+      <c r="S27" s="153"/>
       <c r="T27" s="64"/>
     </row>
     <row r="28" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4414,13 +4422,13 @@
       <c r="J28" s="46"/>
       <c r="K28" s="47"/>
       <c r="L28" s="42"/>
-      <c r="M28" s="191"/>
-      <c r="N28" s="192"/>
-      <c r="O28" s="193"/>
-      <c r="P28" s="194"/>
+      <c r="M28" s="148"/>
+      <c r="N28" s="149"/>
+      <c r="O28" s="150"/>
+      <c r="P28" s="151"/>
       <c r="Q28" s="59"/>
-      <c r="R28" s="189"/>
-      <c r="S28" s="190"/>
+      <c r="R28" s="152"/>
+      <c r="S28" s="153"/>
       <c r="T28" s="64"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4504,12 +4512,12 @@
       <c r="U32" s="2"/>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A33" s="199" t="s">
+      <c r="A33" s="146" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="199"/>
-      <c r="C33" s="199"/>
-      <c r="D33" s="199"/>
+      <c r="B33" s="146"/>
+      <c r="C33" s="146"/>
+      <c r="D33" s="146"/>
       <c r="E33" s="35"/>
       <c r="F33" s="35"/>
       <c r="G33" s="35"/>
@@ -4529,12 +4537,12 @@
       <c r="U33" s="2"/>
     </row>
     <row r="34" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="200" t="s">
+      <c r="A34" s="147" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="200"/>
-      <c r="C34" s="200"/>
-      <c r="D34" s="200"/>
+      <c r="B34" s="147"/>
+      <c r="C34" s="147"/>
+      <c r="D34" s="147"/>
       <c r="E34" s="36"/>
       <c r="F34" s="36"/>
       <c r="G34" s="36"/>
@@ -4577,28 +4585,28 @@
       <c r="U35" s="2"/>
     </row>
     <row r="36" spans="1:21" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="127" t="s">
+      <c r="A36" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="B36" s="127"/>
-      <c r="C36" s="127"/>
-      <c r="D36" s="127"/>
-      <c r="E36" s="127"/>
-      <c r="F36" s="127"/>
-      <c r="G36" s="127"/>
-      <c r="H36" s="127"/>
-      <c r="I36" s="127"/>
-      <c r="J36" s="127"/>
-      <c r="K36" s="127"/>
-      <c r="L36" s="127"/>
-      <c r="M36" s="127"/>
-      <c r="N36" s="127"/>
-      <c r="O36" s="127"/>
-      <c r="P36" s="127"/>
-      <c r="Q36" s="127"/>
-      <c r="R36" s="127"/>
-      <c r="S36" s="127"/>
-      <c r="T36" s="127"/>
+      <c r="B36" s="129"/>
+      <c r="C36" s="129"/>
+      <c r="D36" s="129"/>
+      <c r="E36" s="129"/>
+      <c r="F36" s="129"/>
+      <c r="G36" s="129"/>
+      <c r="H36" s="129"/>
+      <c r="I36" s="129"/>
+      <c r="J36" s="129"/>
+      <c r="K36" s="129"/>
+      <c r="L36" s="129"/>
+      <c r="M36" s="129"/>
+      <c r="N36" s="129"/>
+      <c r="O36" s="129"/>
+      <c r="P36" s="129"/>
+      <c r="Q36" s="129"/>
+      <c r="R36" s="129"/>
+      <c r="S36" s="129"/>
+      <c r="T36" s="129"/>
       <c r="U36" s="2"/>
     </row>
     <row r="37" spans="1:21" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5018,51 +5026,23 @@
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A36:T36"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="R28:S28"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O25:P25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="O23:P23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="R15:S15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="D1:Q4"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="H10:L10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="H11:L11"/>
     <mergeCell ref="M11:Q11"/>
     <mergeCell ref="R11:S14"/>
     <mergeCell ref="T11:T14"/>
@@ -5078,23 +5058,51 @@
     <mergeCell ref="O13:P13"/>
     <mergeCell ref="M14:N14"/>
     <mergeCell ref="O14:P14"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="H10:L10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="B11:B14"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="H11:L11"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="D1:Q4"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="R15:S15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A36:T36"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="R27:S27"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="R28:S28"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.19685039370078741" bottom="0.15748031496062992" header="0" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
chore(verificacion): refresh template visuals
</commit_message>
<xml_diff>
--- a/app/templates/Template_Verificacion.xlsx
+++ b/app/templates/Template_Verificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA5BCF6-4A54-4C9E-81D1-736E25B6FA44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C46904-EB9F-4C2F-AD11-5B27237B0C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A76715E4-29FC-4532-A462-AEFC175FF6CC}"/>
   </bookViews>
@@ -1526,6 +1526,69 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1548,257 +1611,194 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2549,122 +2549,122 @@
     <col min="17" max="17" width="12.44140625" customWidth="1"/>
     <col min="18" max="20" width="10.5546875" customWidth="1"/>
     <col min="21" max="21" width="10.21875" customWidth="1"/>
-    <col min="22" max="22" width="9.6640625" customWidth="1"/>
+    <col min="22" max="22" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="65"/>
       <c r="B1" s="66"/>
       <c r="C1" s="67"/>
-      <c r="D1" s="126" t="s">
+      <c r="D1" s="136" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="126"/>
-      <c r="F1" s="126"/>
-      <c r="G1" s="126"/>
-      <c r="H1" s="126"/>
-      <c r="I1" s="126"/>
-      <c r="J1" s="126"/>
-      <c r="K1" s="126"/>
-      <c r="L1" s="126"/>
-      <c r="M1" s="126"/>
-      <c r="N1" s="126"/>
-      <c r="O1" s="126"/>
-      <c r="P1" s="126"/>
-      <c r="Q1" s="126"/>
-      <c r="R1" s="126"/>
-      <c r="S1" s="126"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="136"/>
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="136"/>
+      <c r="J1" s="136"/>
+      <c r="K1" s="136"/>
+      <c r="L1" s="136"/>
+      <c r="M1" s="136"/>
+      <c r="N1" s="136"/>
+      <c r="O1" s="136"/>
+      <c r="P1" s="136"/>
+      <c r="Q1" s="136"/>
+      <c r="R1" s="136"/>
+      <c r="S1" s="136"/>
       <c r="T1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="U1" s="117" t="s">
+      <c r="U1" s="137" t="s">
         <v>16</v>
       </c>
-      <c r="V1" s="118"/>
+      <c r="V1" s="138"/>
     </row>
     <row r="2" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="68"/>
       <c r="B2" s="4"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="126"/>
-      <c r="Q2" s="126"/>
-      <c r="R2" s="126"/>
-      <c r="S2" s="126"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="136"/>
+      <c r="G2" s="136"/>
+      <c r="H2" s="136"/>
+      <c r="I2" s="136"/>
+      <c r="J2" s="136"/>
+      <c r="K2" s="136"/>
+      <c r="L2" s="136"/>
+      <c r="M2" s="136"/>
+      <c r="N2" s="136"/>
+      <c r="O2" s="136"/>
+      <c r="P2" s="136"/>
+      <c r="Q2" s="136"/>
+      <c r="R2" s="136"/>
+      <c r="S2" s="136"/>
       <c r="T2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="U2" s="119">
+      <c r="U2" s="139">
         <v>3</v>
       </c>
-      <c r="V2" s="120"/>
+      <c r="V2" s="140"/>
     </row>
     <row r="3" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="68"/>
       <c r="B3" s="4"/>
       <c r="C3" s="69"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="126"/>
-      <c r="Q3" s="126"/>
-      <c r="R3" s="126"/>
-      <c r="S3" s="126"/>
+      <c r="D3" s="136"/>
+      <c r="E3" s="136"/>
+      <c r="F3" s="136"/>
+      <c r="G3" s="136"/>
+      <c r="H3" s="136"/>
+      <c r="I3" s="136"/>
+      <c r="J3" s="136"/>
+      <c r="K3" s="136"/>
+      <c r="L3" s="136"/>
+      <c r="M3" s="136"/>
+      <c r="N3" s="136"/>
+      <c r="O3" s="136"/>
+      <c r="P3" s="136"/>
+      <c r="Q3" s="136"/>
+      <c r="R3" s="136"/>
+      <c r="S3" s="136"/>
       <c r="T3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="U3" s="121">
+      <c r="U3" s="141">
         <v>46104</v>
       </c>
-      <c r="V3" s="122"/>
+      <c r="V3" s="142"/>
     </row>
     <row r="4" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="70"/>
       <c r="B4" s="71"/>
       <c r="C4" s="72"/>
-      <c r="D4" s="126"/>
-      <c r="E4" s="126"/>
-      <c r="F4" s="126"/>
-      <c r="G4" s="126"/>
-      <c r="H4" s="126"/>
-      <c r="I4" s="126"/>
-      <c r="J4" s="126"/>
-      <c r="K4" s="126"/>
-      <c r="L4" s="126"/>
-      <c r="M4" s="126"/>
-      <c r="N4" s="126"/>
-      <c r="O4" s="126"/>
-      <c r="P4" s="126"/>
-      <c r="Q4" s="126"/>
-      <c r="R4" s="126"/>
-      <c r="S4" s="126"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="136"/>
+      <c r="F4" s="136"/>
+      <c r="G4" s="136"/>
+      <c r="H4" s="136"/>
+      <c r="I4" s="136"/>
+      <c r="J4" s="136"/>
+      <c r="K4" s="136"/>
+      <c r="L4" s="136"/>
+      <c r="M4" s="136"/>
+      <c r="N4" s="136"/>
+      <c r="O4" s="136"/>
+      <c r="P4" s="136"/>
+      <c r="Q4" s="136"/>
+      <c r="R4" s="136"/>
+      <c r="S4" s="136"/>
       <c r="T4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="U4" s="117" t="s">
+      <c r="U4" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="V4" s="118"/>
+      <c r="V4" s="138"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
@@ -2690,20 +2690,20 @@
       <c r="B6" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="125"/>
-      <c r="D6" s="125"/>
-      <c r="E6" s="125"/>
-      <c r="F6" s="125"/>
-      <c r="G6" s="125"/>
-      <c r="H6" s="125"/>
-      <c r="I6" s="125"/>
-      <c r="J6" s="124" t="s">
+      <c r="C6" s="133"/>
+      <c r="D6" s="133"/>
+      <c r="E6" s="133"/>
+      <c r="F6" s="133"/>
+      <c r="G6" s="133"/>
+      <c r="H6" s="133"/>
+      <c r="I6" s="133"/>
+      <c r="J6" s="132" t="s">
         <v>52</v>
       </c>
-      <c r="K6" s="124"/>
-      <c r="L6" s="124"/>
-      <c r="M6" s="123"/>
-      <c r="N6" s="123"/>
+      <c r="K6" s="132"/>
+      <c r="L6" s="132"/>
+      <c r="M6" s="143"/>
+      <c r="N6" s="143"/>
       <c r="P6" s="76" t="s">
         <v>98</v>
       </c>
@@ -2714,68 +2714,68 @@
       <c r="A7" s="23"/>
       <c r="B7" s="23"/>
       <c r="C7" s="23"/>
-      <c r="D7" s="127"/>
-      <c r="E7" s="127"/>
-      <c r="F7" s="127"/>
-      <c r="G7" s="127"/>
-      <c r="H7" s="128"/>
-      <c r="I7" s="128"/>
-      <c r="J7" s="128"/>
-      <c r="K7" s="128"/>
-      <c r="L7" s="128"/>
+      <c r="D7" s="134"/>
+      <c r="E7" s="134"/>
+      <c r="F7" s="134"/>
+      <c r="G7" s="134"/>
+      <c r="H7" s="135"/>
+      <c r="I7" s="135"/>
+      <c r="J7" s="135"/>
+      <c r="K7" s="135"/>
+      <c r="L7" s="135"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
     </row>
     <row r="8" spans="1:22" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="130" t="s">
+      <c r="A8" s="126" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="130" t="s">
+      <c r="B8" s="126" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="132" t="s">
+      <c r="C8" s="128" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="137" t="s">
+      <c r="D8" s="118" t="s">
         <v>88</v>
       </c>
-      <c r="E8" s="137"/>
-      <c r="F8" s="137"/>
-      <c r="G8" s="137"/>
-      <c r="H8" s="138" t="s">
+      <c r="E8" s="118"/>
+      <c r="F8" s="118"/>
+      <c r="G8" s="118"/>
+      <c r="H8" s="119" t="s">
         <v>67</v>
       </c>
-      <c r="I8" s="139"/>
-      <c r="J8" s="139"/>
-      <c r="K8" s="139"/>
-      <c r="L8" s="140"/>
-      <c r="M8" s="137" t="s">
+      <c r="I8" s="120"/>
+      <c r="J8" s="120"/>
+      <c r="K8" s="120"/>
+      <c r="L8" s="121"/>
+      <c r="M8" s="118" t="s">
         <v>12</v>
       </c>
-      <c r="N8" s="137"/>
-      <c r="O8" s="137"/>
-      <c r="P8" s="134" t="s">
+      <c r="N8" s="118"/>
+      <c r="O8" s="118"/>
+      <c r="P8" s="130" t="s">
         <v>77</v>
       </c>
-      <c r="Q8" s="134" t="s">
+      <c r="Q8" s="130" t="s">
         <v>79</v>
       </c>
-      <c r="R8" s="141" t="s">
+      <c r="R8" s="122" t="s">
         <v>81</v>
       </c>
-      <c r="S8" s="142"/>
-      <c r="T8" s="143"/>
-      <c r="U8" s="136" t="s">
+      <c r="S8" s="123"/>
+      <c r="T8" s="124"/>
+      <c r="U8" s="117" t="s">
         <v>82</v>
       </c>
-      <c r="V8" s="136"/>
+      <c r="V8" s="117"/>
     </row>
     <row r="9" spans="1:22" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="131"/>
-      <c r="B9" s="131"/>
-      <c r="C9" s="133"/>
+      <c r="A9" s="127"/>
+      <c r="B9" s="127"/>
+      <c r="C9" s="129"/>
       <c r="D9" s="87" t="s">
         <v>36</v>
       </c>
@@ -2812,8 +2812,8 @@
       <c r="O9" s="86" t="s">
         <v>96</v>
       </c>
-      <c r="P9" s="135"/>
-      <c r="Q9" s="135"/>
+      <c r="P9" s="131"/>
+      <c r="Q9" s="131"/>
       <c r="R9" s="87" t="s">
         <v>55</v>
       </c>
@@ -2823,8 +2823,8 @@
       <c r="T9" s="87" t="s">
         <v>57</v>
       </c>
-      <c r="U9" s="136"/>
-      <c r="V9" s="136"/>
+      <c r="U9" s="117"/>
+      <c r="V9" s="117"/>
     </row>
     <row r="10" spans="1:22" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="21"/>
@@ -3096,25 +3096,25 @@
       <c r="R20" s="2"/>
     </row>
     <row r="21" spans="1:22" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="129" t="s">
+      <c r="A21" s="125" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="129"/>
-      <c r="C21" s="129"/>
-      <c r="D21" s="129"/>
-      <c r="E21" s="129"/>
-      <c r="F21" s="129"/>
-      <c r="G21" s="129"/>
-      <c r="H21" s="129"/>
-      <c r="I21" s="129"/>
-      <c r="J21" s="129"/>
-      <c r="K21" s="129"/>
-      <c r="L21" s="129"/>
-      <c r="M21" s="129"/>
-      <c r="N21" s="129"/>
-      <c r="O21" s="129"/>
-      <c r="P21" s="129"/>
-      <c r="Q21" s="129"/>
+      <c r="B21" s="125"/>
+      <c r="C21" s="125"/>
+      <c r="D21" s="125"/>
+      <c r="E21" s="125"/>
+      <c r="F21" s="125"/>
+      <c r="G21" s="125"/>
+      <c r="H21" s="125"/>
+      <c r="I21" s="125"/>
+      <c r="J21" s="125"/>
+      <c r="K21" s="125"/>
+      <c r="L21" s="125"/>
+      <c r="M21" s="125"/>
+      <c r="N21" s="125"/>
+      <c r="O21" s="125"/>
+      <c r="P21" s="125"/>
+      <c r="Q21" s="125"/>
       <c r="R21" s="2"/>
     </row>
     <row r="22" spans="1:22" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3483,27 +3483,27 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="U8:V9"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="H8:L8"/>
-    <mergeCell ref="R8:T8"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="U2:V2"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="U4:V4"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="H7:L7"/>
+    <mergeCell ref="D1:S4"/>
     <mergeCell ref="A21:Q21"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="P8:P9"/>
     <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="H7:L7"/>
-    <mergeCell ref="D1:S4"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="U2:V2"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="U4:V4"/>
-    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="U8:V9"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="M8:O8"/>
+    <mergeCell ref="H8:L8"/>
+    <mergeCell ref="R8:T8"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.19685039370078741" header="0" footer="0"/>
@@ -3657,110 +3657,110 @@
       <c r="A1" s="65"/>
       <c r="B1" s="66"/>
       <c r="C1" s="67"/>
-      <c r="D1" s="196" t="s">
+      <c r="D1" s="146" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="197"/>
-      <c r="F1" s="197"/>
-      <c r="G1" s="197"/>
-      <c r="H1" s="197"/>
-      <c r="I1" s="197"/>
-      <c r="J1" s="197"/>
-      <c r="K1" s="197"/>
-      <c r="L1" s="197"/>
-      <c r="M1" s="197"/>
-      <c r="N1" s="197"/>
-      <c r="O1" s="197"/>
-      <c r="P1" s="197"/>
-      <c r="Q1" s="198"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="147"/>
+      <c r="K1" s="147"/>
+      <c r="L1" s="147"/>
+      <c r="M1" s="147"/>
+      <c r="N1" s="147"/>
+      <c r="O1" s="147"/>
+      <c r="P1" s="147"/>
+      <c r="Q1" s="148"/>
       <c r="R1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="S1" s="117" t="s">
+      <c r="S1" s="137" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="118"/>
+      <c r="T1" s="138"/>
       <c r="U1" s="1"/>
     </row>
     <row r="2" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="68"/>
       <c r="B2" s="4"/>
       <c r="C2" s="69"/>
-      <c r="D2" s="199"/>
-      <c r="E2" s="200"/>
-      <c r="F2" s="200"/>
-      <c r="G2" s="200"/>
-      <c r="H2" s="200"/>
-      <c r="I2" s="200"/>
-      <c r="J2" s="200"/>
-      <c r="K2" s="200"/>
-      <c r="L2" s="200"/>
-      <c r="M2" s="200"/>
-      <c r="N2" s="200"/>
-      <c r="O2" s="200"/>
-      <c r="P2" s="200"/>
-      <c r="Q2" s="201"/>
+      <c r="D2" s="149"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="150"/>
+      <c r="G2" s="150"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="150"/>
+      <c r="J2" s="150"/>
+      <c r="K2" s="150"/>
+      <c r="L2" s="150"/>
+      <c r="M2" s="150"/>
+      <c r="N2" s="150"/>
+      <c r="O2" s="150"/>
+      <c r="P2" s="150"/>
+      <c r="Q2" s="151"/>
       <c r="R2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="S2" s="117">
+      <c r="S2" s="137">
         <v>1</v>
       </c>
-      <c r="T2" s="118"/>
+      <c r="T2" s="138"/>
       <c r="U2" s="1"/>
     </row>
     <row r="3" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="68"/>
       <c r="B3" s="4"/>
       <c r="C3" s="69"/>
-      <c r="D3" s="199"/>
-      <c r="E3" s="200"/>
-      <c r="F3" s="200"/>
-      <c r="G3" s="200"/>
-      <c r="H3" s="200"/>
-      <c r="I3" s="200"/>
-      <c r="J3" s="200"/>
-      <c r="K3" s="200"/>
-      <c r="L3" s="200"/>
-      <c r="M3" s="200"/>
-      <c r="N3" s="200"/>
-      <c r="O3" s="200"/>
-      <c r="P3" s="200"/>
-      <c r="Q3" s="201"/>
+      <c r="D3" s="149"/>
+      <c r="E3" s="150"/>
+      <c r="F3" s="150"/>
+      <c r="G3" s="150"/>
+      <c r="H3" s="150"/>
+      <c r="I3" s="150"/>
+      <c r="J3" s="150"/>
+      <c r="K3" s="150"/>
+      <c r="L3" s="150"/>
+      <c r="M3" s="150"/>
+      <c r="N3" s="150"/>
+      <c r="O3" s="150"/>
+      <c r="P3" s="150"/>
+      <c r="Q3" s="151"/>
       <c r="R3" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="S3" s="117">
+      <c r="S3" s="137">
         <v>45232</v>
       </c>
-      <c r="T3" s="118"/>
+      <c r="T3" s="138"/>
       <c r="U3" s="1"/>
     </row>
     <row r="4" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="70"/>
       <c r="B4" s="71"/>
       <c r="C4" s="72"/>
-      <c r="D4" s="202"/>
-      <c r="E4" s="203"/>
-      <c r="F4" s="203"/>
-      <c r="G4" s="203"/>
-      <c r="H4" s="203"/>
-      <c r="I4" s="203"/>
-      <c r="J4" s="203"/>
-      <c r="K4" s="203"/>
-      <c r="L4" s="203"/>
-      <c r="M4" s="203"/>
-      <c r="N4" s="203"/>
-      <c r="O4" s="203"/>
-      <c r="P4" s="203"/>
-      <c r="Q4" s="204"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="153"/>
+      <c r="F4" s="153"/>
+      <c r="G4" s="153"/>
+      <c r="H4" s="153"/>
+      <c r="I4" s="153"/>
+      <c r="J4" s="153"/>
+      <c r="K4" s="153"/>
+      <c r="L4" s="153"/>
+      <c r="M4" s="153"/>
+      <c r="N4" s="153"/>
+      <c r="O4" s="153"/>
+      <c r="P4" s="153"/>
+      <c r="Q4" s="154"/>
       <c r="R4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="S4" s="117" t="s">
+      <c r="S4" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="T4" s="118"/>
+      <c r="T4" s="138"/>
       <c r="U4" s="1"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -3793,16 +3793,16 @@
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
       <c r="D6" s="27"/>
-      <c r="E6" s="192"/>
-      <c r="F6" s="192"/>
+      <c r="E6" s="155"/>
+      <c r="F6" s="155"/>
       <c r="G6" s="28"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="193" t="s">
+      <c r="J6" s="156" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="193"/>
-      <c r="L6" s="193"/>
+      <c r="K6" s="156"/>
+      <c r="L6" s="156"/>
       <c r="M6" s="33"/>
       <c r="N6" s="52"/>
       <c r="O6" s="33"/>
@@ -3820,11 +3820,11 @@
       <c r="D7" s="18"/>
       <c r="E7" s="9"/>
       <c r="F7" s="10"/>
-      <c r="G7" s="194"/>
-      <c r="H7" s="194"/>
-      <c r="I7" s="194"/>
-      <c r="J7" s="194"/>
-      <c r="K7" s="194"/>
+      <c r="G7" s="157"/>
+      <c r="H7" s="157"/>
+      <c r="I7" s="157"/>
+      <c r="J7" s="157"/>
+      <c r="K7" s="157"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -3838,10 +3838,10 @@
       <c r="B8" s="23"/>
       <c r="C8" s="23"/>
       <c r="D8" s="29"/>
-      <c r="E8" s="195"/>
-      <c r="F8" s="195"/>
-      <c r="G8" s="195"/>
-      <c r="H8" s="195"/>
+      <c r="E8" s="158"/>
+      <c r="F8" s="158"/>
+      <c r="G8" s="158"/>
+      <c r="H8" s="158"/>
       <c r="I8" s="34"/>
       <c r="J8" s="34"/>
       <c r="K8" s="34"/>
@@ -3861,10 +3861,10 @@
       <c r="B9" s="23"/>
       <c r="C9" s="23"/>
       <c r="D9" s="29"/>
-      <c r="E9" s="195"/>
-      <c r="F9" s="195"/>
-      <c r="G9" s="195"/>
-      <c r="H9" s="195"/>
+      <c r="E9" s="158"/>
+      <c r="F9" s="158"/>
+      <c r="G9" s="158"/>
+      <c r="H9" s="158"/>
       <c r="I9" s="34"/>
       <c r="J9" s="34"/>
       <c r="K9" s="34"/>
@@ -3880,19 +3880,19 @@
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>
-      <c r="D10" s="127" t="s">
+      <c r="D10" s="134" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="127"/>
-      <c r="F10" s="127"/>
-      <c r="G10" s="127"/>
-      <c r="H10" s="128" t="s">
+      <c r="E10" s="134"/>
+      <c r="F10" s="134"/>
+      <c r="G10" s="134"/>
+      <c r="H10" s="135" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="128"/>
-      <c r="J10" s="128"/>
-      <c r="K10" s="128"/>
-      <c r="L10" s="128"/>
+      <c r="I10" s="135"/>
+      <c r="J10" s="135"/>
+      <c r="K10" s="135"/>
+      <c r="L10" s="135"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
@@ -3900,116 +3900,116 @@
       <c r="U10" s="1"/>
     </row>
     <row r="11" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="184" t="s">
+      <c r="A11" s="159" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="185" t="s">
+      <c r="B11" s="160" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="178" t="s">
+      <c r="C11" s="161" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="187" t="s">
+      <c r="D11" s="164" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="188"/>
-      <c r="F11" s="188"/>
-      <c r="G11" s="189"/>
-      <c r="H11" s="190" t="s">
+      <c r="E11" s="165"/>
+      <c r="F11" s="165"/>
+      <c r="G11" s="166"/>
+      <c r="H11" s="167" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="191"/>
-      <c r="J11" s="191"/>
-      <c r="K11" s="191"/>
-      <c r="L11" s="191"/>
-      <c r="M11" s="160" t="s">
+      <c r="I11" s="168"/>
+      <c r="J11" s="168"/>
+      <c r="K11" s="168"/>
+      <c r="L11" s="168"/>
+      <c r="M11" s="169" t="s">
         <v>18</v>
       </c>
-      <c r="N11" s="161"/>
-      <c r="O11" s="161"/>
-      <c r="P11" s="161"/>
-      <c r="Q11" s="161"/>
-      <c r="R11" s="162" t="s">
+      <c r="N11" s="170"/>
+      <c r="O11" s="170"/>
+      <c r="P11" s="170"/>
+      <c r="Q11" s="170"/>
+      <c r="R11" s="171" t="s">
         <v>34</v>
       </c>
-      <c r="S11" s="163"/>
-      <c r="T11" s="168" t="s">
+      <c r="S11" s="172"/>
+      <c r="T11" s="177" t="s">
         <v>33</v>
       </c>
       <c r="U11" s="1"/>
     </row>
     <row r="12" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="184"/>
-      <c r="B12" s="185"/>
-      <c r="C12" s="186"/>
-      <c r="D12" s="170" t="s">
+      <c r="A12" s="159"/>
+      <c r="B12" s="160"/>
+      <c r="C12" s="162"/>
+      <c r="D12" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="171"/>
-      <c r="F12" s="171"/>
-      <c r="G12" s="172"/>
-      <c r="H12" s="170" t="s">
+      <c r="E12" s="180"/>
+      <c r="F12" s="180"/>
+      <c r="G12" s="181"/>
+      <c r="H12" s="179" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="171"/>
-      <c r="J12" s="171"/>
-      <c r="K12" s="171"/>
-      <c r="L12" s="172"/>
-      <c r="M12" s="170" t="s">
+      <c r="I12" s="180"/>
+      <c r="J12" s="180"/>
+      <c r="K12" s="180"/>
+      <c r="L12" s="181"/>
+      <c r="M12" s="179" t="s">
         <v>12</v>
       </c>
-      <c r="N12" s="171"/>
-      <c r="O12" s="171"/>
-      <c r="P12" s="171"/>
-      <c r="Q12" s="171"/>
-      <c r="R12" s="164"/>
-      <c r="S12" s="165"/>
-      <c r="T12" s="169"/>
+      <c r="N12" s="180"/>
+      <c r="O12" s="180"/>
+      <c r="P12" s="180"/>
+      <c r="Q12" s="180"/>
+      <c r="R12" s="173"/>
+      <c r="S12" s="174"/>
+      <c r="T12" s="178"/>
     </row>
     <row r="13" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="184"/>
-      <c r="B13" s="185"/>
-      <c r="C13" s="186"/>
-      <c r="D13" s="173" t="s">
+      <c r="A13" s="159"/>
+      <c r="B13" s="160"/>
+      <c r="C13" s="162"/>
+      <c r="D13" s="182" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="136" t="s">
+      <c r="E13" s="117" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="174" t="s">
+      <c r="F13" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="175"/>
-      <c r="H13" s="176" t="s">
+      <c r="G13" s="184"/>
+      <c r="H13" s="185" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="177"/>
-      <c r="J13" s="177"/>
-      <c r="K13" s="177"/>
-      <c r="L13" s="178" t="s">
+      <c r="I13" s="186"/>
+      <c r="J13" s="186"/>
+      <c r="K13" s="186"/>
+      <c r="L13" s="161" t="s">
         <v>41</v>
       </c>
-      <c r="M13" s="180" t="s">
+      <c r="M13" s="187" t="s">
         <v>24</v>
       </c>
-      <c r="N13" s="181"/>
-      <c r="O13" s="182" t="s">
+      <c r="N13" s="188"/>
+      <c r="O13" s="189" t="s">
         <v>25</v>
       </c>
-      <c r="P13" s="182"/>
+      <c r="P13" s="189"/>
       <c r="Q13" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="R13" s="164"/>
-      <c r="S13" s="165"/>
-      <c r="T13" s="169"/>
+      <c r="R13" s="173"/>
+      <c r="S13" s="174"/>
+      <c r="T13" s="178"/>
     </row>
     <row r="14" spans="1:21" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="184"/>
-      <c r="B14" s="185"/>
-      <c r="C14" s="179"/>
-      <c r="D14" s="173"/>
-      <c r="E14" s="136"/>
+      <c r="A14" s="159"/>
+      <c r="B14" s="160"/>
+      <c r="C14" s="163"/>
+      <c r="D14" s="182"/>
+      <c r="E14" s="117"/>
       <c r="F14" s="62" t="s">
         <v>28</v>
       </c>
@@ -4028,21 +4028,21 @@
       <c r="K14" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="L14" s="179"/>
-      <c r="M14" s="183" t="s">
+      <c r="L14" s="163"/>
+      <c r="M14" s="190" t="s">
         <v>23</v>
       </c>
-      <c r="N14" s="139"/>
-      <c r="O14" s="138" t="s">
+      <c r="N14" s="120"/>
+      <c r="O14" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="P14" s="140"/>
+      <c r="P14" s="121"/>
       <c r="Q14" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="R14" s="166"/>
-      <c r="S14" s="167"/>
-      <c r="T14" s="169"/>
+      <c r="R14" s="175"/>
+      <c r="S14" s="176"/>
+      <c r="T14" s="178"/>
     </row>
     <row r="15" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="21">
@@ -4077,13 +4077,13 @@
       <c r="L15" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="M15" s="158"/>
-      <c r="N15" s="159"/>
-      <c r="O15" s="158"/>
-      <c r="P15" s="159"/>
+      <c r="M15" s="191"/>
+      <c r="N15" s="192"/>
+      <c r="O15" s="191"/>
+      <c r="P15" s="192"/>
       <c r="Q15" s="58"/>
-      <c r="R15" s="152"/>
-      <c r="S15" s="153"/>
+      <c r="R15" s="193"/>
+      <c r="S15" s="194"/>
       <c r="T15" s="64"/>
     </row>
     <row r="16" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4104,21 +4104,21 @@
       <c r="J16" s="46"/>
       <c r="K16" s="47"/>
       <c r="L16" s="42"/>
-      <c r="M16" s="148" t="s">
+      <c r="M16" s="195" t="s">
         <v>44</v>
       </c>
-      <c r="N16" s="149"/>
-      <c r="O16" s="150" t="s">
+      <c r="N16" s="196"/>
+      <c r="O16" s="197" t="s">
         <v>44</v>
       </c>
-      <c r="P16" s="151"/>
+      <c r="P16" s="198"/>
       <c r="Q16" s="58" t="s">
         <v>46</v>
       </c>
-      <c r="R16" s="152" t="s">
+      <c r="R16" s="193" t="s">
         <v>15</v>
       </c>
-      <c r="S16" s="153"/>
+      <c r="S16" s="194"/>
       <c r="T16" s="64" t="s">
         <v>15</v>
       </c>
@@ -4138,21 +4138,21 @@
       <c r="J17" s="46"/>
       <c r="K17" s="47"/>
       <c r="L17" s="42"/>
-      <c r="M17" s="148" t="s">
+      <c r="M17" s="195" t="s">
         <v>45</v>
       </c>
-      <c r="N17" s="149"/>
-      <c r="O17" s="150" t="s">
+      <c r="N17" s="196"/>
+      <c r="O17" s="197" t="s">
         <v>46</v>
       </c>
-      <c r="P17" s="151"/>
+      <c r="P17" s="198"/>
       <c r="Q17" s="74" t="s">
         <v>53</v>
       </c>
-      <c r="R17" s="154" t="s">
+      <c r="R17" s="199" t="s">
         <v>48</v>
       </c>
-      <c r="S17" s="155"/>
+      <c r="S17" s="200"/>
       <c r="T17" s="64" t="s">
         <v>46</v>
       </c>
@@ -4172,21 +4172,21 @@
       <c r="J18" s="46"/>
       <c r="K18" s="47"/>
       <c r="L18" s="42"/>
-      <c r="M18" s="148" t="s">
+      <c r="M18" s="195" t="s">
         <v>45</v>
       </c>
-      <c r="N18" s="149"/>
-      <c r="O18" s="150" t="s">
+      <c r="N18" s="196"/>
+      <c r="O18" s="197" t="s">
         <v>46</v>
       </c>
-      <c r="P18" s="151"/>
+      <c r="P18" s="198"/>
       <c r="Q18" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="R18" s="156" t="s">
+      <c r="R18" s="201" t="s">
         <v>47</v>
       </c>
-      <c r="S18" s="157"/>
+      <c r="S18" s="202"/>
       <c r="T18" s="64" t="s">
         <v>46</v>
       </c>
@@ -4206,13 +4206,13 @@
       <c r="J19" s="46"/>
       <c r="K19" s="47"/>
       <c r="L19" s="42"/>
-      <c r="M19" s="148"/>
-      <c r="N19" s="149"/>
-      <c r="O19" s="150"/>
-      <c r="P19" s="151"/>
+      <c r="M19" s="195"/>
+      <c r="N19" s="196"/>
+      <c r="O19" s="197"/>
+      <c r="P19" s="198"/>
       <c r="Q19" s="58"/>
-      <c r="R19" s="152"/>
-      <c r="S19" s="153"/>
+      <c r="R19" s="193"/>
+      <c r="S19" s="194"/>
       <c r="T19" s="64"/>
     </row>
     <row r="20" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4230,13 +4230,13 @@
       <c r="J20" s="46"/>
       <c r="K20" s="47"/>
       <c r="L20" s="42"/>
-      <c r="M20" s="148"/>
-      <c r="N20" s="149"/>
-      <c r="O20" s="150"/>
-      <c r="P20" s="151"/>
+      <c r="M20" s="195"/>
+      <c r="N20" s="196"/>
+      <c r="O20" s="197"/>
+      <c r="P20" s="198"/>
       <c r="Q20" s="58"/>
-      <c r="R20" s="152"/>
-      <c r="S20" s="153"/>
+      <c r="R20" s="193"/>
+      <c r="S20" s="194"/>
       <c r="T20" s="64"/>
     </row>
     <row r="21" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4254,13 +4254,13 @@
       <c r="J21" s="46"/>
       <c r="K21" s="47"/>
       <c r="L21" s="42"/>
-      <c r="M21" s="148"/>
-      <c r="N21" s="149"/>
-      <c r="O21" s="150"/>
-      <c r="P21" s="151"/>
+      <c r="M21" s="195"/>
+      <c r="N21" s="196"/>
+      <c r="O21" s="197"/>
+      <c r="P21" s="198"/>
       <c r="Q21" s="58"/>
-      <c r="R21" s="152"/>
-      <c r="S21" s="153"/>
+      <c r="R21" s="193"/>
+      <c r="S21" s="194"/>
       <c r="T21" s="64"/>
     </row>
     <row r="22" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4278,13 +4278,13 @@
       <c r="J22" s="46"/>
       <c r="K22" s="47"/>
       <c r="L22" s="42"/>
-      <c r="M22" s="148"/>
-      <c r="N22" s="149"/>
-      <c r="O22" s="150"/>
-      <c r="P22" s="151"/>
+      <c r="M22" s="195"/>
+      <c r="N22" s="196"/>
+      <c r="O22" s="197"/>
+      <c r="P22" s="198"/>
       <c r="Q22" s="58"/>
-      <c r="R22" s="152"/>
-      <c r="S22" s="153"/>
+      <c r="R22" s="193"/>
+      <c r="S22" s="194"/>
       <c r="T22" s="64"/>
     </row>
     <row r="23" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4302,13 +4302,13 @@
       <c r="J23" s="46"/>
       <c r="K23" s="47"/>
       <c r="L23" s="42"/>
-      <c r="M23" s="148"/>
-      <c r="N23" s="149"/>
-      <c r="O23" s="150"/>
-      <c r="P23" s="151"/>
+      <c r="M23" s="195"/>
+      <c r="N23" s="196"/>
+      <c r="O23" s="197"/>
+      <c r="P23" s="198"/>
       <c r="Q23" s="58"/>
-      <c r="R23" s="152"/>
-      <c r="S23" s="153"/>
+      <c r="R23" s="193"/>
+      <c r="S23" s="194"/>
       <c r="T23" s="64"/>
     </row>
     <row r="24" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4326,13 +4326,13 @@
       <c r="J24" s="46"/>
       <c r="K24" s="47"/>
       <c r="L24" s="42"/>
-      <c r="M24" s="148"/>
-      <c r="N24" s="149"/>
-      <c r="O24" s="150"/>
-      <c r="P24" s="151"/>
+      <c r="M24" s="195"/>
+      <c r="N24" s="196"/>
+      <c r="O24" s="197"/>
+      <c r="P24" s="198"/>
       <c r="Q24" s="58"/>
-      <c r="R24" s="152"/>
-      <c r="S24" s="153"/>
+      <c r="R24" s="193"/>
+      <c r="S24" s="194"/>
       <c r="T24" s="64"/>
     </row>
     <row r="25" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4350,13 +4350,13 @@
       <c r="J25" s="46"/>
       <c r="K25" s="47"/>
       <c r="L25" s="42"/>
-      <c r="M25" s="148"/>
-      <c r="N25" s="149"/>
-      <c r="O25" s="150"/>
-      <c r="P25" s="151"/>
+      <c r="M25" s="195"/>
+      <c r="N25" s="196"/>
+      <c r="O25" s="197"/>
+      <c r="P25" s="198"/>
       <c r="Q25" s="58"/>
-      <c r="R25" s="152"/>
-      <c r="S25" s="153"/>
+      <c r="R25" s="193"/>
+      <c r="S25" s="194"/>
       <c r="T25" s="64"/>
     </row>
     <row r="26" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4374,13 +4374,13 @@
       <c r="J26" s="46"/>
       <c r="K26" s="47"/>
       <c r="L26" s="42"/>
-      <c r="M26" s="148"/>
-      <c r="N26" s="149"/>
-      <c r="O26" s="150"/>
-      <c r="P26" s="151"/>
+      <c r="M26" s="195"/>
+      <c r="N26" s="196"/>
+      <c r="O26" s="197"/>
+      <c r="P26" s="198"/>
       <c r="Q26" s="58"/>
-      <c r="R26" s="152"/>
-      <c r="S26" s="153"/>
+      <c r="R26" s="193"/>
+      <c r="S26" s="194"/>
       <c r="T26" s="64"/>
     </row>
     <row r="27" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4398,13 +4398,13 @@
       <c r="J27" s="46"/>
       <c r="K27" s="47"/>
       <c r="L27" s="42"/>
-      <c r="M27" s="148"/>
-      <c r="N27" s="149"/>
-      <c r="O27" s="150"/>
-      <c r="P27" s="151"/>
+      <c r="M27" s="195"/>
+      <c r="N27" s="196"/>
+      <c r="O27" s="197"/>
+      <c r="P27" s="198"/>
       <c r="Q27" s="58"/>
-      <c r="R27" s="152"/>
-      <c r="S27" s="153"/>
+      <c r="R27" s="193"/>
+      <c r="S27" s="194"/>
       <c r="T27" s="64"/>
     </row>
     <row r="28" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4422,13 +4422,13 @@
       <c r="J28" s="46"/>
       <c r="K28" s="47"/>
       <c r="L28" s="42"/>
-      <c r="M28" s="148"/>
-      <c r="N28" s="149"/>
-      <c r="O28" s="150"/>
-      <c r="P28" s="151"/>
+      <c r="M28" s="195"/>
+      <c r="N28" s="196"/>
+      <c r="O28" s="197"/>
+      <c r="P28" s="198"/>
       <c r="Q28" s="59"/>
-      <c r="R28" s="152"/>
-      <c r="S28" s="153"/>
+      <c r="R28" s="193"/>
+      <c r="S28" s="194"/>
       <c r="T28" s="64"/>
     </row>
     <row r="29" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4512,12 +4512,12 @@
       <c r="U32" s="2"/>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A33" s="146" t="s">
+      <c r="A33" s="203" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="146"/>
-      <c r="C33" s="146"/>
-      <c r="D33" s="146"/>
+      <c r="B33" s="203"/>
+      <c r="C33" s="203"/>
+      <c r="D33" s="203"/>
       <c r="E33" s="35"/>
       <c r="F33" s="35"/>
       <c r="G33" s="35"/>
@@ -4537,12 +4537,12 @@
       <c r="U33" s="2"/>
     </row>
     <row r="34" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="147" t="s">
+      <c r="A34" s="204" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="147"/>
-      <c r="C34" s="147"/>
-      <c r="D34" s="147"/>
+      <c r="B34" s="204"/>
+      <c r="C34" s="204"/>
+      <c r="D34" s="204"/>
       <c r="E34" s="36"/>
       <c r="F34" s="36"/>
       <c r="G34" s="36"/>
@@ -4585,28 +4585,28 @@
       <c r="U35" s="2"/>
     </row>
     <row r="36" spans="1:21" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="129" t="s">
+      <c r="A36" s="125" t="s">
         <v>8</v>
       </c>
-      <c r="B36" s="129"/>
-      <c r="C36" s="129"/>
-      <c r="D36" s="129"/>
-      <c r="E36" s="129"/>
-      <c r="F36" s="129"/>
-      <c r="G36" s="129"/>
-      <c r="H36" s="129"/>
-      <c r="I36" s="129"/>
-      <c r="J36" s="129"/>
-      <c r="K36" s="129"/>
-      <c r="L36" s="129"/>
-      <c r="M36" s="129"/>
-      <c r="N36" s="129"/>
-      <c r="O36" s="129"/>
-      <c r="P36" s="129"/>
-      <c r="Q36" s="129"/>
-      <c r="R36" s="129"/>
-      <c r="S36" s="129"/>
-      <c r="T36" s="129"/>
+      <c r="B36" s="125"/>
+      <c r="C36" s="125"/>
+      <c r="D36" s="125"/>
+      <c r="E36" s="125"/>
+      <c r="F36" s="125"/>
+      <c r="G36" s="125"/>
+      <c r="H36" s="125"/>
+      <c r="I36" s="125"/>
+      <c r="J36" s="125"/>
+      <c r="K36" s="125"/>
+      <c r="L36" s="125"/>
+      <c r="M36" s="125"/>
+      <c r="N36" s="125"/>
+      <c r="O36" s="125"/>
+      <c r="P36" s="125"/>
+      <c r="Q36" s="125"/>
+      <c r="R36" s="125"/>
+      <c r="S36" s="125"/>
+      <c r="T36" s="125"/>
       <c r="U36" s="2"/>
     </row>
     <row r="37" spans="1:21" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5026,23 +5026,51 @@
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="D1:Q4"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="H10:L10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="B11:B14"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="H11:L11"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A36:T36"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="R27:S27"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="R15:S15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="R16:S16"/>
     <mergeCell ref="M11:Q11"/>
     <mergeCell ref="R11:S14"/>
     <mergeCell ref="T11:T14"/>
@@ -5058,51 +5086,23 @@
     <mergeCell ref="O13:P13"/>
     <mergeCell ref="M14:N14"/>
     <mergeCell ref="O14:P14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="R15:S15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="R16:S16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="O23:P23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="O25:P25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A36:T36"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="O27:P27"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="H10:L10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="H11:L11"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="D1:Q4"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="S4:T4"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.19685039370078741" bottom="0.15748031496062992" header="0" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
chore: actualizar template verificacion
</commit_message>
<xml_diff>
--- a/app/templates/Template_Verificacion.xlsx
+++ b/app/templates/Template_Verificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C46904-EB9F-4C2F-AD11-5B27237B0C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6B7970-F77C-45BF-822E-57C08921F58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A76715E4-29FC-4532-A462-AEFC175FF6CC}"/>
   </bookViews>
@@ -2606,7 +2606,7 @@
         <v>1</v>
       </c>
       <c r="U2" s="139">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V2" s="140"/>
     </row>
@@ -2634,7 +2634,7 @@
         <v>3</v>
       </c>
       <c r="U3" s="141">
-        <v>46104</v>
+        <v>46070</v>
       </c>
       <c r="V3" s="142"/>
     </row>

</xml_diff>